<commit_message>
Normativa de octubre 2026 (PDF del alumno), IVA retenido sin crédito fiscal, cotización del empleador sin doble conteo del SIS
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012WV3i5CNskdg7dgJ6kwcHp
</commit_message>
<xml_diff>
--- a/trabajo_juan_castillo/cambio_sujeto_silvestres.xlsx
+++ b/trabajo_juan_castillo/cambio_sujeto_silvestres.xlsx
@@ -617,7 +617,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="171" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="421">
+  <cellXfs count="422">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1835,8 +1835,11 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="10" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="1">
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="10" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+      <protection locked="1" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="14" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="1" hidden="1"/>
     </xf>
     <xf numFmtId="3" fontId="9" fillId="5" borderId="10" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="1">
@@ -2780,7 +2783,7 @@
       </c>
       <c r="M11" s="6" t="n"/>
       <c r="N11" s="31">
-        <f>O5</f>
+        <f>O5+K31</f>
         <v/>
       </c>
       <c r="O11" s="1" t="n"/>
@@ -2871,9 +2874,8 @@
         </is>
       </c>
       <c r="M15" s="6" t="n"/>
-      <c r="N15" s="31">
-        <f>I31</f>
-        <v/>
+      <c r="N15" s="31" t="n">
+        <v>0</v>
       </c>
       <c r="O15" s="1" t="n"/>
     </row>
@@ -3506,7 +3508,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Las facturas de compra (DTE 46) las emite el comprador; el crédito fiscal es el IVA total y el IVA retenido se paga en el F29.</t>
+          <t>Las facturas de compra (DTE 46) las emite el comprador; el IVA retenido total no da derecho a crédito fiscal y se paga en el F29 (reverso, código 39).</t>
         </is>
       </c>
       <c r="F66" s="98" t="n"/>
@@ -4634,9 +4636,8 @@
         <v/>
       </c>
       <c r="C75" s="6" t="n"/>
-      <c r="D75" s="38">
-        <f>'L. COMPRAS'!I64</f>
-        <v/>
+      <c r="D75" s="38" t="n">
+        <v>0</v>
       </c>
       <c r="E75" s="6" t="n"/>
       <c r="G75" s="325" t="inlineStr">
@@ -7297,62 +7298,68 @@
       <c r="A34" s="8" t="n"/>
       <c r="B34" s="351" t="n"/>
       <c r="C34" s="352" t="n"/>
-      <c r="D34" s="146" t="n">
+      <c r="D34" s="356" t="n">
         <v>22</v>
       </c>
-      <c r="E34" s="355" t="n"/>
-      <c r="F34" s="204" t="inlineStr">
+      <c r="E34" s="357" t="n"/>
+      <c r="F34" s="376" t="inlineStr">
         <is>
           <t>Sin Derecho a Credito Fiscal</t>
         </is>
       </c>
-      <c r="G34" s="342" t="n"/>
-      <c r="H34" s="152" t="inlineStr">
+      <c r="G34" s="377" t="n"/>
+      <c r="H34" s="358" t="inlineStr">
         <is>
           <t>Internas afectas</t>
         </is>
       </c>
-      <c r="I34" s="339" t="n"/>
-      <c r="J34" s="339" t="n"/>
-      <c r="K34" s="339" t="n"/>
-      <c r="L34" s="339" t="n"/>
-      <c r="M34" s="339" t="n"/>
-      <c r="N34" s="339" t="n"/>
-      <c r="O34" s="339" t="n"/>
-      <c r="P34" s="339" t="n"/>
-      <c r="Q34" s="339" t="n"/>
-      <c r="R34" s="339" t="n"/>
-      <c r="S34" s="339" t="n"/>
-      <c r="T34" s="339" t="n"/>
-      <c r="U34" s="339" t="n"/>
-      <c r="V34" s="340" t="n"/>
-      <c r="W34" s="153" t="n">
+      <c r="I34" s="359" t="n"/>
+      <c r="J34" s="359" t="n"/>
+      <c r="K34" s="359" t="n"/>
+      <c r="L34" s="359" t="n"/>
+      <c r="M34" s="359" t="n"/>
+      <c r="N34" s="359" t="n"/>
+      <c r="O34" s="359" t="n"/>
+      <c r="P34" s="359" t="n"/>
+      <c r="Q34" s="359" t="n"/>
+      <c r="R34" s="359" t="n"/>
+      <c r="S34" s="359" t="n"/>
+      <c r="T34" s="359" t="n"/>
+      <c r="U34" s="359" t="n"/>
+      <c r="V34" s="360" t="n"/>
+      <c r="W34" s="361" t="n">
         <v>564</v>
       </c>
-      <c r="X34" s="340" t="n"/>
-      <c r="Y34" s="369" t="n"/>
-      <c r="Z34" s="349" t="n"/>
-      <c r="AA34" s="349" t="n"/>
-      <c r="AB34" s="349" t="n"/>
-      <c r="AC34" s="349" t="n"/>
-      <c r="AD34" s="349" t="n"/>
-      <c r="AE34" s="349" t="n"/>
-      <c r="AF34" s="349" t="n"/>
-      <c r="AG34" s="349" t="n"/>
-      <c r="AH34" s="349" t="n"/>
-      <c r="AI34" s="349" t="n"/>
-      <c r="AJ34" s="349" t="n"/>
-      <c r="AK34" s="349" t="n"/>
-      <c r="AL34" s="349" t="n"/>
-      <c r="AM34" s="350" t="n"/>
-      <c r="AN34" s="155" t="n">
+      <c r="X34" s="360" t="n"/>
+      <c r="Y34" s="371">
+        <f>COUNT('L. COMPRAS'!B7:B30)</f>
+        <v/>
+      </c>
+      <c r="Z34" s="363" t="n"/>
+      <c r="AA34" s="363" t="n"/>
+      <c r="AB34" s="363" t="n"/>
+      <c r="AC34" s="363" t="n"/>
+      <c r="AD34" s="363" t="n"/>
+      <c r="AE34" s="363" t="n"/>
+      <c r="AF34" s="363" t="n"/>
+      <c r="AG34" s="363" t="n"/>
+      <c r="AH34" s="363" t="n"/>
+      <c r="AI34" s="363" t="n"/>
+      <c r="AJ34" s="363" t="n"/>
+      <c r="AK34" s="363" t="n"/>
+      <c r="AL34" s="363" t="n"/>
+      <c r="AM34" s="364" t="n"/>
+      <c r="AN34" s="356" t="n">
         <v>521</v>
       </c>
-      <c r="AO34" s="340" t="n"/>
-      <c r="AP34" s="353" t="n"/>
-      <c r="AQ34" s="349" t="n"/>
-      <c r="AR34" s="350" t="n"/>
-      <c r="AS34" s="146" t="n"/>
+      <c r="AO34" s="360" t="n"/>
+      <c r="AP34" s="378">
+        <f>'L. COMPRAS'!H31</f>
+        <v/>
+      </c>
+      <c r="AQ34" s="363" t="n"/>
+      <c r="AR34" s="364" t="n"/>
+      <c r="AS34" s="356" t="n"/>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="8" t="n"/>
@@ -7527,72 +7534,66 @@
       <c r="A38" s="8" t="n"/>
       <c r="B38" s="351" t="n"/>
       <c r="C38" s="352" t="n"/>
-      <c r="D38" s="356" t="n">
+      <c r="D38" s="146" t="n">
         <v>25</v>
       </c>
-      <c r="E38" s="357" t="n"/>
-      <c r="F38" s="376" t="inlineStr">
+      <c r="E38" s="355" t="n"/>
+      <c r="F38" s="209" t="inlineStr">
         <is>
           <t>Con Derecho a Crédito Fiscal</t>
         </is>
       </c>
-      <c r="G38" s="376" t="inlineStr">
+      <c r="G38" s="209" t="inlineStr">
         <is>
           <t>Internas</t>
         </is>
       </c>
-      <c r="H38" s="358" t="inlineStr">
+      <c r="H38" s="152" t="inlineStr">
         <is>
           <t>Facturas recibidas del giro y Facturas de compra emitidas</t>
         </is>
       </c>
-      <c r="I38" s="359" t="n"/>
-      <c r="J38" s="359" t="n"/>
-      <c r="K38" s="359" t="n"/>
-      <c r="L38" s="359" t="n"/>
-      <c r="M38" s="359" t="n"/>
-      <c r="N38" s="359" t="n"/>
-      <c r="O38" s="359" t="n"/>
-      <c r="P38" s="359" t="n"/>
-      <c r="Q38" s="359" t="n"/>
-      <c r="R38" s="359" t="n"/>
-      <c r="S38" s="359" t="n"/>
-      <c r="T38" s="359" t="n"/>
-      <c r="U38" s="359" t="n"/>
-      <c r="V38" s="360" t="n"/>
-      <c r="W38" s="361" t="n">
+      <c r="I38" s="339" t="n"/>
+      <c r="J38" s="339" t="n"/>
+      <c r="K38" s="339" t="n"/>
+      <c r="L38" s="339" t="n"/>
+      <c r="M38" s="339" t="n"/>
+      <c r="N38" s="339" t="n"/>
+      <c r="O38" s="339" t="n"/>
+      <c r="P38" s="339" t="n"/>
+      <c r="Q38" s="339" t="n"/>
+      <c r="R38" s="339" t="n"/>
+      <c r="S38" s="339" t="n"/>
+      <c r="T38" s="339" t="n"/>
+      <c r="U38" s="339" t="n"/>
+      <c r="V38" s="340" t="n"/>
+      <c r="W38" s="153" t="n">
         <v>519</v>
       </c>
-      <c r="X38" s="360" t="n"/>
-      <c r="Y38" s="371">
-        <f>COUNT('L. COMPRAS'!B7:B30)</f>
-        <v/>
-      </c>
-      <c r="Z38" s="363" t="n"/>
-      <c r="AA38" s="363" t="n"/>
-      <c r="AB38" s="363" t="n"/>
-      <c r="AC38" s="363" t="n"/>
-      <c r="AD38" s="363" t="n"/>
-      <c r="AE38" s="363" t="n"/>
-      <c r="AF38" s="363" t="n"/>
-      <c r="AG38" s="363" t="n"/>
-      <c r="AH38" s="363" t="n"/>
-      <c r="AI38" s="363" t="n"/>
-      <c r="AJ38" s="363" t="n"/>
-      <c r="AK38" s="363" t="n"/>
-      <c r="AL38" s="363" t="n"/>
-      <c r="AM38" s="364" t="n"/>
-      <c r="AN38" s="356" t="n">
+      <c r="X38" s="340" t="n"/>
+      <c r="Y38" s="369" t="n"/>
+      <c r="Z38" s="349" t="n"/>
+      <c r="AA38" s="349" t="n"/>
+      <c r="AB38" s="349" t="n"/>
+      <c r="AC38" s="349" t="n"/>
+      <c r="AD38" s="349" t="n"/>
+      <c r="AE38" s="349" t="n"/>
+      <c r="AF38" s="349" t="n"/>
+      <c r="AG38" s="349" t="n"/>
+      <c r="AH38" s="349" t="n"/>
+      <c r="AI38" s="349" t="n"/>
+      <c r="AJ38" s="349" t="n"/>
+      <c r="AK38" s="349" t="n"/>
+      <c r="AL38" s="349" t="n"/>
+      <c r="AM38" s="350" t="n"/>
+      <c r="AN38" s="155" t="n">
         <v>520</v>
       </c>
-      <c r="AO38" s="360" t="n"/>
-      <c r="AP38" s="377">
-        <f>'L. COMPRAS'!I31</f>
-        <v/>
-      </c>
-      <c r="AQ38" s="363" t="n"/>
-      <c r="AR38" s="364" t="n"/>
-      <c r="AS38" s="372" t="inlineStr">
+      <c r="AO38" s="340" t="n"/>
+      <c r="AP38" s="353" t="n"/>
+      <c r="AQ38" s="349" t="n"/>
+      <c r="AR38" s="350" t="n"/>
+      <c r="AS38" s="89" t="inlineStr">
         <is>
           <t>+</t>
         </is>
@@ -7608,7 +7609,7 @@
       <c r="E39" s="355" t="n"/>
       <c r="F39" s="355" t="n"/>
       <c r="G39" s="355" t="n"/>
-      <c r="H39" s="378" t="inlineStr">
+      <c r="H39" s="379" t="inlineStr">
         <is>
           <t>Facturas activo fijo</t>
         </is>
@@ -7631,7 +7632,7 @@
         <v>524</v>
       </c>
       <c r="X39" s="340" t="n"/>
-      <c r="Y39" s="379" t="n"/>
+      <c r="Y39" s="380" t="n"/>
       <c r="Z39" s="349" t="n"/>
       <c r="AA39" s="349" t="n"/>
       <c r="AB39" s="349" t="n"/>
@@ -7650,7 +7651,7 @@
         <v>525</v>
       </c>
       <c r="AO39" s="340" t="n"/>
-      <c r="AP39" s="380" t="n"/>
+      <c r="AP39" s="381" t="n"/>
       <c r="AQ39" s="349" t="n"/>
       <c r="AR39" s="350" t="n"/>
       <c r="AS39" s="89" t="inlineStr">
@@ -7730,7 +7731,7 @@
       <c r="E41" s="355" t="n"/>
       <c r="F41" s="355" t="n"/>
       <c r="G41" s="347" t="n"/>
-      <c r="H41" s="378" t="inlineStr">
+      <c r="H41" s="379" t="inlineStr">
         <is>
           <t>Notas de Débito recibidas</t>
         </is>
@@ -7753,7 +7754,7 @@
         <v>531</v>
       </c>
       <c r="X41" s="340" t="n"/>
-      <c r="Y41" s="379" t="n"/>
+      <c r="Y41" s="380" t="n"/>
       <c r="Z41" s="349" t="n"/>
       <c r="AA41" s="349" t="n"/>
       <c r="AB41" s="349" t="n"/>
@@ -7790,7 +7791,7 @@
       </c>
       <c r="E42" s="355" t="n"/>
       <c r="F42" s="355" t="n"/>
-      <c r="G42" s="381" t="inlineStr">
+      <c r="G42" s="382" t="inlineStr">
         <is>
           <t>Impor-tación</t>
         </is>
@@ -7914,7 +7915,7 @@
       <c r="D44" s="155" t="n">
         <v>31</v>
       </c>
-      <c r="E44" s="378" t="inlineStr">
+      <c r="E44" s="379" t="inlineStr">
         <is>
           <t>Remanente Crédito Fiscal del mes anterior</t>
         </is>
@@ -8333,29 +8334,29 @@
           <t>M3 Comprados con derecho a crédito</t>
         </is>
       </c>
-      <c r="S51" s="382" t="n"/>
-      <c r="T51" s="382" t="n"/>
-      <c r="U51" s="382" t="n"/>
-      <c r="V51" s="382" t="n"/>
-      <c r="W51" s="382" t="n"/>
-      <c r="X51" s="382" t="n"/>
-      <c r="Y51" s="382" t="n"/>
-      <c r="Z51" s="383" t="n"/>
+      <c r="S51" s="383" t="n"/>
+      <c r="T51" s="383" t="n"/>
+      <c r="U51" s="383" t="n"/>
+      <c r="V51" s="383" t="n"/>
+      <c r="W51" s="383" t="n"/>
+      <c r="X51" s="383" t="n"/>
+      <c r="Y51" s="383" t="n"/>
+      <c r="Z51" s="384" t="n"/>
       <c r="AC51" s="278" t="inlineStr">
         <is>
           <t>Componentes del Impuesto</t>
         </is>
       </c>
-      <c r="AD51" s="382" t="n"/>
-      <c r="AE51" s="382" t="n"/>
-      <c r="AF51" s="382" t="n"/>
-      <c r="AG51" s="382" t="n"/>
-      <c r="AH51" s="382" t="n"/>
-      <c r="AI51" s="382" t="n"/>
-      <c r="AJ51" s="382" t="n"/>
-      <c r="AK51" s="382" t="n"/>
-      <c r="AL51" s="382" t="n"/>
-      <c r="AM51" s="383" t="n"/>
+      <c r="AD51" s="383" t="n"/>
+      <c r="AE51" s="383" t="n"/>
+      <c r="AF51" s="383" t="n"/>
+      <c r="AG51" s="383" t="n"/>
+      <c r="AH51" s="383" t="n"/>
+      <c r="AI51" s="383" t="n"/>
+      <c r="AJ51" s="383" t="n"/>
+      <c r="AK51" s="383" t="n"/>
+      <c r="AL51" s="383" t="n"/>
+      <c r="AM51" s="384" t="n"/>
       <c r="AN51" s="155" t="n"/>
       <c r="AO51" s="340" t="n"/>
       <c r="AP51" s="353" t="n"/>
@@ -8370,7 +8371,7 @@
       <c r="D52" s="146" t="n">
         <v>38</v>
       </c>
-      <c r="E52" s="384" t="inlineStr">
+      <c r="E52" s="385" t="inlineStr">
         <is>
           <t>Recuperación  del Impto. Específico al Petróleo Diesel (Art. 7º Ley 18.502 y 3º D.S. Nº 311/86)</t>
         </is>
@@ -8422,8 +8423,8 @@
       </c>
       <c r="AO52" s="342" t="n"/>
       <c r="AP52" s="375" t="n"/>
-      <c r="AQ52" s="385" t="n"/>
-      <c r="AR52" s="386" t="n"/>
+      <c r="AQ52" s="386" t="n"/>
+      <c r="AR52" s="387" t="n"/>
       <c r="AS52" s="24" t="inlineStr">
         <is>
           <t>+</t>
@@ -8478,9 +8479,9 @@
       <c r="AM53" s="340" t="n"/>
       <c r="AN53" s="344" t="n"/>
       <c r="AO53" s="346" t="n"/>
-      <c r="AP53" s="387" t="n"/>
-      <c r="AQ53" s="388" t="n"/>
-      <c r="AR53" s="389" t="n"/>
+      <c r="AP53" s="388" t="n"/>
+      <c r="AQ53" s="389" t="n"/>
+      <c r="AR53" s="390" t="n"/>
       <c r="AS53" s="347" t="n"/>
     </row>
     <row r="54" ht="27.75" customHeight="1">
@@ -8490,7 +8491,7 @@
       <c r="D54" s="146" t="n">
         <v>39</v>
       </c>
-      <c r="E54" s="384" t="inlineStr">
+      <c r="E54" s="385" t="inlineStr">
         <is>
           <t>Recuperación  del Impto. Específico al Petróleo Diesel soportado por Transportistas de Carga (Art. 2º Ley 19.764)</t>
         </is>
@@ -8542,8 +8543,8 @@
       </c>
       <c r="AO54" s="342" t="n"/>
       <c r="AP54" s="375" t="n"/>
-      <c r="AQ54" s="385" t="n"/>
-      <c r="AR54" s="386" t="n"/>
+      <c r="AQ54" s="386" t="n"/>
+      <c r="AR54" s="387" t="n"/>
       <c r="AS54" s="24" t="inlineStr">
         <is>
           <t>+</t>
@@ -8598,9 +8599,9 @@
       <c r="AM55" s="340" t="n"/>
       <c r="AN55" s="344" t="n"/>
       <c r="AO55" s="346" t="n"/>
-      <c r="AP55" s="387" t="n"/>
-      <c r="AQ55" s="388" t="n"/>
-      <c r="AR55" s="389" t="n"/>
+      <c r="AP55" s="388" t="n"/>
+      <c r="AQ55" s="389" t="n"/>
+      <c r="AR55" s="390" t="n"/>
       <c r="AS55" s="347" t="n"/>
     </row>
     <row r="56" ht="27.75" customHeight="1">
@@ -8610,7 +8611,7 @@
       <c r="D56" s="146" t="n">
         <v>40</v>
       </c>
-      <c r="E56" s="390" t="inlineStr">
+      <c r="E56" s="391" t="inlineStr">
         <is>
           <t>Crédito del Art. 11º Ley 18.211 (correspondiente a Zona Franca de Extensión)</t>
         </is>
@@ -8826,9 +8827,9 @@
       <c r="AN59" s="8" t="n"/>
       <c r="AO59" s="8" t="n"/>
       <c r="AP59" s="8" t="n"/>
-      <c r="AQ59" s="391" t="n"/>
-      <c r="AR59" s="392" t="n"/>
-      <c r="AS59" s="392" t="n"/>
+      <c r="AQ59" s="392" t="n"/>
+      <c r="AR59" s="393" t="n"/>
+      <c r="AS59" s="393" t="n"/>
     </row>
     <row r="60" ht="15.75" customHeight="1">
       <c r="A60" s="8" t="n"/>
@@ -9005,7 +9006,7 @@
         <v>77</v>
       </c>
       <c r="Q63" s="340" t="n"/>
-      <c r="R63" s="393" t="n"/>
+      <c r="R63" s="394" t="n"/>
       <c r="S63" s="349" t="n"/>
       <c r="T63" s="349" t="n"/>
       <c r="U63" s="349" t="n"/>
@@ -9035,7 +9036,7 @@
         <v>89</v>
       </c>
       <c r="AO63" s="340" t="n"/>
-      <c r="AP63" s="394">
+      <c r="AP63" s="395">
         <f>MAX(AP29-AP58,0)</f>
         <v/>
       </c>
@@ -9228,7 +9229,7 @@
         <v>46</v>
       </c>
       <c r="E67" s="355" t="n"/>
-      <c r="F67" s="378" t="inlineStr">
+      <c r="F67" s="379" t="inlineStr">
         <is>
           <t>Retención de Impuesto con tasa del 10% sobre las rentas del Art. 42 Nº2, según Art. 74 Nº2 LIR</t>
         </is>
@@ -9630,7 +9631,7 @@
       <c r="AK73" s="339" t="n"/>
       <c r="AL73" s="339" t="n"/>
       <c r="AM73" s="340" t="n"/>
-      <c r="AN73" s="395" t="inlineStr">
+      <c r="AN73" s="396" t="inlineStr">
         <is>
           <t>PPM Neto Determinado</t>
         </is>
@@ -9663,7 +9664,7 @@
       <c r="I74" s="175" t="n">
         <v>30</v>
       </c>
-      <c r="J74" s="396" t="n"/>
+      <c r="J74" s="397" t="n"/>
       <c r="K74" s="349" t="n"/>
       <c r="L74" s="349" t="n"/>
       <c r="M74" s="349" t="n"/>
@@ -9674,7 +9675,7 @@
       <c r="R74" s="153" t="n">
         <v>563</v>
       </c>
-      <c r="S74" s="397">
+      <c r="S74" s="398">
         <f>'L. VENTAS'!C81</f>
         <v/>
       </c>
@@ -9689,7 +9690,7 @@
         <v>115</v>
       </c>
       <c r="AB74" s="340" t="n"/>
-      <c r="AC74" s="398">
+      <c r="AC74" s="399">
         <f>'L. VENTAS'!A81</f>
         <v/>
       </c>
@@ -9698,7 +9699,7 @@
         <v>68</v>
       </c>
       <c r="AF74" s="340" t="n"/>
-      <c r="AG74" s="399" t="n"/>
+      <c r="AG74" s="400" t="n"/>
       <c r="AH74" s="349" t="n"/>
       <c r="AI74" s="349" t="n"/>
       <c r="AJ74" s="349" t="n"/>
@@ -9709,7 +9710,7 @@
         <v>62</v>
       </c>
       <c r="AO74" s="340" t="n"/>
-      <c r="AP74" s="400">
+      <c r="AP74" s="401">
         <f>'L. VENTAS'!D81</f>
         <v/>
       </c>
@@ -9739,7 +9740,7 @@
       <c r="I75" s="175" t="n">
         <v>565</v>
       </c>
-      <c r="J75" s="396" t="n"/>
+      <c r="J75" s="397" t="n"/>
       <c r="K75" s="349" t="n"/>
       <c r="L75" s="349" t="n"/>
       <c r="M75" s="349" t="n"/>
@@ -9750,7 +9751,7 @@
       <c r="R75" s="175" t="n">
         <v>120</v>
       </c>
-      <c r="S75" s="401" t="n"/>
+      <c r="S75" s="402" t="n"/>
       <c r="T75" s="349" t="n"/>
       <c r="U75" s="349" t="n"/>
       <c r="V75" s="349" t="n"/>
@@ -9762,13 +9763,13 @@
         <v>542</v>
       </c>
       <c r="AB75" s="340" t="n"/>
-      <c r="AC75" s="398" t="n"/>
+      <c r="AC75" s="399" t="n"/>
       <c r="AD75" s="350" t="n"/>
       <c r="AE75" s="175" t="n">
         <v>122</v>
       </c>
       <c r="AF75" s="340" t="n"/>
-      <c r="AG75" s="399" t="n"/>
+      <c r="AG75" s="400" t="n"/>
       <c r="AH75" s="349" t="n"/>
       <c r="AI75" s="349" t="n"/>
       <c r="AJ75" s="349" t="n"/>
@@ -9806,7 +9807,7 @@
       <c r="I76" s="175" t="n">
         <v>700</v>
       </c>
-      <c r="J76" s="396" t="n"/>
+      <c r="J76" s="397" t="n"/>
       <c r="K76" s="349" t="n"/>
       <c r="L76" s="349" t="n"/>
       <c r="M76" s="349" t="n"/>
@@ -9817,7 +9818,7 @@
       <c r="R76" s="175" t="n">
         <v>701</v>
       </c>
-      <c r="S76" s="401" t="n"/>
+      <c r="S76" s="402" t="n"/>
       <c r="T76" s="349" t="n"/>
       <c r="U76" s="349" t="n"/>
       <c r="V76" s="349" t="n"/>
@@ -9829,13 +9830,13 @@
         <v>702</v>
       </c>
       <c r="AB76" s="340" t="n"/>
-      <c r="AC76" s="398" t="n"/>
+      <c r="AC76" s="399" t="n"/>
       <c r="AD76" s="350" t="n"/>
       <c r="AE76" s="175" t="n">
         <v>711</v>
       </c>
       <c r="AF76" s="340" t="n"/>
-      <c r="AG76" s="399" t="n"/>
+      <c r="AG76" s="400" t="n"/>
       <c r="AH76" s="349" t="n"/>
       <c r="AI76" s="349" t="n"/>
       <c r="AJ76" s="349" t="n"/>
@@ -9922,56 +9923,56 @@
         <v>56</v>
       </c>
       <c r="E78" s="355" t="n"/>
-      <c r="F78" s="402" t="inlineStr">
+      <c r="F78" s="403" t="inlineStr">
         <is>
           <t>Crédito Capacitación</t>
         </is>
       </c>
-      <c r="G78" s="403" t="n"/>
-      <c r="H78" s="404" t="n"/>
+      <c r="G78" s="404" t="n"/>
+      <c r="H78" s="405" t="n"/>
       <c r="I78" s="278" t="inlineStr">
         <is>
           <t>Crédito del mes</t>
         </is>
       </c>
-      <c r="J78" s="382" t="n"/>
-      <c r="K78" s="382" t="n"/>
-      <c r="L78" s="382" t="n"/>
-      <c r="M78" s="382" t="n"/>
-      <c r="N78" s="382" t="n"/>
-      <c r="O78" s="382" t="n"/>
-      <c r="P78" s="382" t="n"/>
-      <c r="Q78" s="383" t="n"/>
+      <c r="J78" s="383" t="n"/>
+      <c r="K78" s="383" t="n"/>
+      <c r="L78" s="383" t="n"/>
+      <c r="M78" s="383" t="n"/>
+      <c r="N78" s="383" t="n"/>
+      <c r="O78" s="383" t="n"/>
+      <c r="P78" s="383" t="n"/>
+      <c r="Q78" s="384" t="n"/>
       <c r="R78" s="278" t="inlineStr">
         <is>
           <t>Remanente mes Anterior</t>
         </is>
       </c>
-      <c r="S78" s="382" t="n"/>
-      <c r="T78" s="382" t="n"/>
-      <c r="U78" s="382" t="n"/>
-      <c r="V78" s="382" t="n"/>
-      <c r="W78" s="382" t="n"/>
-      <c r="X78" s="382" t="n"/>
-      <c r="Y78" s="382" t="n"/>
-      <c r="Z78" s="383" t="n"/>
+      <c r="S78" s="383" t="n"/>
+      <c r="T78" s="383" t="n"/>
+      <c r="U78" s="383" t="n"/>
+      <c r="V78" s="383" t="n"/>
+      <c r="W78" s="383" t="n"/>
+      <c r="X78" s="383" t="n"/>
+      <c r="Y78" s="383" t="n"/>
+      <c r="Z78" s="384" t="n"/>
       <c r="AA78" s="278" t="inlineStr">
         <is>
           <t>Remanente Período sgte</t>
         </is>
       </c>
-      <c r="AB78" s="382" t="n"/>
-      <c r="AC78" s="382" t="n"/>
-      <c r="AD78" s="382" t="n"/>
-      <c r="AE78" s="382" t="n"/>
-      <c r="AF78" s="382" t="n"/>
-      <c r="AG78" s="383" t="n"/>
+      <c r="AB78" s="383" t="n"/>
+      <c r="AC78" s="383" t="n"/>
+      <c r="AD78" s="383" t="n"/>
+      <c r="AE78" s="383" t="n"/>
+      <c r="AF78" s="383" t="n"/>
+      <c r="AG78" s="384" t="n"/>
       <c r="AH78" s="278" t="n"/>
-      <c r="AI78" s="382" t="n"/>
-      <c r="AJ78" s="382" t="n"/>
-      <c r="AK78" s="382" t="n"/>
-      <c r="AL78" s="382" t="n"/>
-      <c r="AM78" s="383" t="n"/>
+      <c r="AI78" s="383" t="n"/>
+      <c r="AJ78" s="383" t="n"/>
+      <c r="AK78" s="383" t="n"/>
+      <c r="AL78" s="383" t="n"/>
+      <c r="AM78" s="384" t="n"/>
       <c r="AN78" s="146" t="n"/>
       <c r="AO78" s="340" t="n"/>
       <c r="AP78" s="353" t="n"/>
@@ -9985,13 +9986,13 @@
       <c r="C79" s="352" t="n"/>
       <c r="D79" s="355" t="n"/>
       <c r="E79" s="355" t="n"/>
-      <c r="F79" s="405" t="inlineStr">
+      <c r="F79" s="406" t="inlineStr">
         <is>
           <t>Ley 19.518/97</t>
         </is>
       </c>
-      <c r="G79" s="406" t="n"/>
-      <c r="H79" s="407" t="n"/>
+      <c r="G79" s="407" t="n"/>
+      <c r="H79" s="408" t="n"/>
       <c r="I79" s="175" t="n">
         <v>721</v>
       </c>
@@ -10017,7 +10018,7 @@
       <c r="AA79" s="278" t="n">
         <v>724</v>
       </c>
-      <c r="AB79" s="383" t="n"/>
+      <c r="AB79" s="384" t="n"/>
       <c r="AC79" s="99" t="n"/>
       <c r="AD79" s="99" t="n"/>
       <c r="AE79" s="99" t="n"/>
@@ -10028,11 +10029,11 @@
           <t>Crédito a imutar</t>
         </is>
       </c>
-      <c r="AI79" s="403" t="n"/>
-      <c r="AJ79" s="403" t="n"/>
-      <c r="AK79" s="403" t="n"/>
-      <c r="AL79" s="403" t="n"/>
-      <c r="AM79" s="404" t="n"/>
+      <c r="AI79" s="404" t="n"/>
+      <c r="AJ79" s="404" t="n"/>
+      <c r="AK79" s="404" t="n"/>
+      <c r="AL79" s="404" t="n"/>
+      <c r="AM79" s="405" t="n"/>
       <c r="AN79" s="155" t="n">
         <v>723</v>
       </c>
@@ -10261,7 +10262,7 @@
         <v>595</v>
       </c>
       <c r="AO83" s="340" t="n"/>
-      <c r="AP83" s="400">
+      <c r="AP83" s="401">
         <f>AP63+AP74</f>
         <v/>
       </c>
@@ -10322,7 +10323,7 @@
     </row>
     <row r="85" ht="15.75" customHeight="1">
       <c r="A85" s="8" t="n"/>
-      <c r="B85" s="390" t="inlineStr">
+      <c r="B85" s="391" t="inlineStr">
         <is>
           <t xml:space="preserve">Si no declara Tributación Simplificada, Impuesto Adicional (Art. 37 o Art. 42), Cotización Adicional, Crédito Especial Empresas Constructoras, Recuperación de Peaje Transportistas de Pasajeros o Cambio de Sujeto; traslade el valor a línea 47 (código 595) </t>
         </is>
@@ -10474,7 +10475,7 @@
           <t>05</t>
         </is>
       </c>
-      <c r="AJ87" s="395" t="inlineStr">
+      <c r="AJ87" s="396" t="inlineStr">
         <is>
           <t>Nombres</t>
         </is>
@@ -10491,7 +10492,7 @@
     </row>
     <row r="88" ht="23.25" customHeight="1">
       <c r="A88" s="8" t="n"/>
-      <c r="B88" s="408" t="inlineStr">
+      <c r="B88" s="409" t="inlineStr">
         <is>
           <t>Silvestres del Ñuble SpA (ficticia)</t>
         </is>
@@ -10558,8 +10559,8 @@
       <c r="K89" s="146" t="n">
         <v>583</v>
       </c>
-      <c r="L89" s="409" t="n"/>
-      <c r="M89" s="410" t="n"/>
+      <c r="L89" s="410" t="n"/>
+      <c r="M89" s="411" t="n"/>
       <c r="N89" s="8" t="n"/>
       <c r="O89" s="8" t="n"/>
       <c r="P89" s="8" t="n"/>
@@ -10609,8 +10610,8 @@
       <c r="I90" s="345" t="n"/>
       <c r="J90" s="346" t="n"/>
       <c r="K90" s="347" t="n"/>
-      <c r="L90" s="411" t="n"/>
-      <c r="M90" s="412" t="n"/>
+      <c r="L90" s="412" t="n"/>
+      <c r="M90" s="413" t="n"/>
       <c r="N90" s="8" t="inlineStr">
         <is>
           <t>(Si marca con X el casillero, registre los cambios al reverso)</t>
@@ -10697,7 +10698,7 @@
     </row>
     <row r="92" ht="18.75" customHeight="1">
       <c r="A92" s="8" t="n"/>
-      <c r="B92" s="390" t="inlineStr">
+      <c r="B92" s="391" t="inlineStr">
         <is>
           <t>Declaro bajo juramento que los datos contenidos en esta declaración son la expresión fiel de la verdad, por lo que asumo la responsabilidad correspondiente.</t>
         </is>
@@ -10749,7 +10750,7 @@
         <v>91</v>
       </c>
       <c r="AO92" s="340" t="n"/>
-      <c r="AP92" s="400">
+      <c r="AP92" s="401">
         <f>AP83+AP100</f>
         <v/>
       </c>
@@ -10764,17 +10765,17 @@
     <row r="93" ht="18.75" customHeight="1">
       <c r="A93" s="8" t="n"/>
       <c r="B93" s="351" t="n"/>
-      <c r="C93" s="392" t="n"/>
-      <c r="D93" s="392" t="n"/>
-      <c r="E93" s="392" t="n"/>
-      <c r="F93" s="392" t="n"/>
-      <c r="G93" s="392" t="n"/>
-      <c r="H93" s="392" t="n"/>
-      <c r="I93" s="392" t="n"/>
-      <c r="J93" s="392" t="n"/>
-      <c r="K93" s="392" t="n"/>
-      <c r="L93" s="392" t="n"/>
-      <c r="M93" s="392" t="n"/>
+      <c r="C93" s="393" t="n"/>
+      <c r="D93" s="393" t="n"/>
+      <c r="E93" s="393" t="n"/>
+      <c r="F93" s="393" t="n"/>
+      <c r="G93" s="393" t="n"/>
+      <c r="H93" s="393" t="n"/>
+      <c r="I93" s="393" t="n"/>
+      <c r="J93" s="393" t="n"/>
+      <c r="K93" s="393" t="n"/>
+      <c r="L93" s="393" t="n"/>
+      <c r="M93" s="393" t="n"/>
       <c r="N93" s="352" t="n"/>
       <c r="O93" s="8" t="n"/>
       <c r="P93" s="8" t="n"/>
@@ -10987,7 +10988,7 @@
     <row r="102">
       <c r="B102" t="inlineStr">
         <is>
-          <t>Amarillo: línea 5 (retención total, vendedor retenido), líneas 6 y 14 (retención parcial, vendedor retenido) y línea 25 (facturas de compra emitidas por el comprador: crédito fiscal).</t>
+          <t>Amarillo: línea 5 (retención total, vendedor retenido), líneas 6 y 14 (retención parcial, vendedor retenido) y línea 22 (compras sin derecho a crédito fiscal: la factura de compra del agente retenedor, códigos 564 y 521).</t>
         </is>
       </c>
     </row>
@@ -11407,7 +11408,7 @@
       <c r="E2" s="6" t="n"/>
     </row>
     <row r="3" ht="18.75" customHeight="1">
-      <c r="B3" s="413" t="n"/>
+      <c r="B3" s="414" t="n"/>
       <c r="C3" s="315" t="n">
         <v>2024</v>
       </c>
@@ -11640,7 +11641,7 @@
           <t>Empresa (ficticia)</t>
         </is>
       </c>
-      <c r="B1" s="414" t="inlineStr">
+      <c r="B1" s="415" t="inlineStr">
         <is>
           <t>Silvestres del Ñuble SpA (ficticia)</t>
         </is>
@@ -11652,7 +11653,7 @@
           <t>RUT (ficticio)</t>
         </is>
       </c>
-      <c r="B2" s="414" t="inlineStr">
+      <c r="B2" s="415" t="inlineStr">
         <is>
           <t>76.123.456-0</t>
         </is>
@@ -11664,7 +11665,7 @@
           <t>Período</t>
         </is>
       </c>
-      <c r="B3" s="414" t="inlineStr">
+      <c r="B3" s="415" t="inlineStr">
         <is>
           <t>Octubre 2026</t>
         </is>
@@ -11676,7 +11677,7 @@
           <t>Tasa de IVA</t>
         </is>
       </c>
-      <c r="B4" s="415" t="n">
+      <c r="B4" s="416" t="n">
         <v>0.19</v>
       </c>
     </row>
@@ -11686,7 +11687,7 @@
           <t>Retención del IVA (1 = total; Res. Ex. SII 4095/2000)</t>
         </is>
       </c>
-      <c r="B5" s="415" t="n">
+      <c r="B5" s="416" t="n">
         <v>1</v>
       </c>
     </row>
@@ -11696,7 +11697,7 @@
           <t>Margen de ganancia sobre el costo</t>
         </is>
       </c>
-      <c r="B6" s="415" t="n">
+      <c r="B6" s="416" t="n">
         <v>0.4</v>
       </c>
     </row>
@@ -11706,7 +11707,7 @@
           <t>Integrantes</t>
         </is>
       </c>
-      <c r="B7" s="414" t="inlineStr">
+      <c r="B7" s="415" t="inlineStr">
         <is>
           <t>Matius Loyola, Diego Quintana, Joaquín Verdejo</t>
         </is>
@@ -11755,93 +11756,93 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="416" t="inlineStr">
+      <c r="A4" s="417" t="inlineStr">
         <is>
           <t>Folio</t>
         </is>
       </c>
-      <c r="B4" s="416" t="inlineStr">
+      <c r="B4" s="417" t="inlineStr">
         <is>
           <t>Fecha</t>
         </is>
       </c>
-      <c r="C4" s="416" t="inlineStr">
+      <c r="C4" s="417" t="inlineStr">
         <is>
           <t>Proveedor</t>
         </is>
       </c>
-      <c r="D4" s="416" t="inlineStr">
+      <c r="D4" s="417" t="inlineStr">
         <is>
           <t>RUT</t>
         </is>
       </c>
-      <c r="E4" s="416" t="inlineStr">
+      <c r="E4" s="417" t="inlineStr">
         <is>
           <t>Producto</t>
         </is>
       </c>
-      <c r="F4" s="416" t="inlineStr">
+      <c r="F4" s="417" t="inlineStr">
         <is>
           <t>Kilos</t>
         </is>
       </c>
-      <c r="G4" s="416" t="inlineStr">
+      <c r="G4" s="417" t="inlineStr">
         <is>
           <t>Precio por kilo</t>
         </is>
       </c>
-      <c r="H4" s="416" t="inlineStr">
+      <c r="H4" s="417" t="inlineStr">
         <is>
           <t>Neto</t>
         </is>
       </c>
-      <c r="I4" s="416" t="inlineStr">
+      <c r="I4" s="417" t="inlineStr">
         <is>
           <t>IVA 19 %</t>
         </is>
       </c>
-      <c r="J4" s="416" t="inlineStr">
+      <c r="J4" s="417" t="inlineStr">
         <is>
           <t>IVA retenido</t>
         </is>
       </c>
-      <c r="K4" s="416" t="inlineStr">
+      <c r="K4" s="417" t="inlineStr">
         <is>
           <t>IVA que cobra el proveedor</t>
         </is>
       </c>
-      <c r="L4" s="416" t="inlineStr">
+      <c r="L4" s="417" t="inlineStr">
         <is>
           <t>Total a pagar al proveedor</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="414" t="n">
+      <c r="A5" s="415" t="n">
         <v>201</v>
       </c>
-      <c r="B5" s="417" t="n">
+      <c r="B5" s="418" t="n">
         <v>46297</v>
       </c>
-      <c r="C5" s="414" t="inlineStr">
+      <c r="C5" s="415" t="inlineStr">
         <is>
           <t>Juan Pérez (recolector)</t>
         </is>
       </c>
-      <c r="D5" s="414" t="inlineStr">
+      <c r="D5" s="415" t="inlineStr">
         <is>
           <t>11.111.111-1</t>
         </is>
       </c>
-      <c r="E5" s="414" t="inlineStr">
+      <c r="E5" s="415" t="inlineStr">
         <is>
           <t>Rosa mosqueta</t>
         </is>
       </c>
-      <c r="F5" s="418" t="n">
+      <c r="F5" s="419" t="n">
         <v>1200</v>
       </c>
-      <c r="G5" s="418" t="n">
+      <c r="G5" s="419" t="n">
         <v>1500</v>
       </c>
       <c r="H5" s="47">
@@ -11866,31 +11867,31 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="414" t="n">
+      <c r="A6" s="415" t="n">
         <v>202</v>
       </c>
-      <c r="B6" s="417" t="n">
+      <c r="B6" s="418" t="n">
         <v>46301</v>
       </c>
-      <c r="C6" s="414" t="inlineStr">
+      <c r="C6" s="415" t="inlineStr">
         <is>
           <t>María Soto (recolectora)</t>
         </is>
       </c>
-      <c r="D6" s="414" t="inlineStr">
+      <c r="D6" s="415" t="inlineStr">
         <is>
           <t>12.222.222-5</t>
         </is>
       </c>
-      <c r="E6" s="414" t="inlineStr">
+      <c r="E6" s="415" t="inlineStr">
         <is>
           <t>Hongos</t>
         </is>
       </c>
-      <c r="F6" s="418" t="n">
+      <c r="F6" s="419" t="n">
         <v>300</v>
       </c>
-      <c r="G6" s="418" t="n">
+      <c r="G6" s="419" t="n">
         <v>4000</v>
       </c>
       <c r="H6" s="47">
@@ -11915,31 +11916,31 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="414" t="n">
+      <c r="A7" s="415" t="n">
         <v>203</v>
       </c>
-      <c r="B7" s="417" t="n">
+      <c r="B7" s="418" t="n">
         <v>46307</v>
       </c>
-      <c r="C7" s="414" t="inlineStr">
+      <c r="C7" s="415" t="inlineStr">
         <is>
           <t>Pedro Núñez (recolector)</t>
         </is>
       </c>
-      <c r="D7" s="414" t="inlineStr">
+      <c r="D7" s="415" t="inlineStr">
         <is>
           <t>13.333.333-9</t>
         </is>
       </c>
-      <c r="E7" s="414" t="inlineStr">
+      <c r="E7" s="415" t="inlineStr">
         <is>
           <t>Mora</t>
         </is>
       </c>
-      <c r="F7" s="418" t="n">
+      <c r="F7" s="419" t="n">
         <v>500</v>
       </c>
-      <c r="G7" s="418" t="n">
+      <c r="G7" s="419" t="n">
         <v>1600</v>
       </c>
       <c r="H7" s="47">
@@ -11964,31 +11965,31 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="414" t="n">
+      <c r="A8" s="415" t="n">
         <v>204</v>
       </c>
-      <c r="B8" s="417" t="n">
+      <c r="B8" s="418" t="n">
         <v>46314</v>
       </c>
-      <c r="C8" s="414" t="inlineStr">
+      <c r="C8" s="415" t="inlineStr">
         <is>
           <t>Rosa Muñoz (recolectora)</t>
         </is>
       </c>
-      <c r="D8" s="414" t="inlineStr">
+      <c r="D8" s="415" t="inlineStr">
         <is>
           <t>14.444.444-2</t>
         </is>
       </c>
-      <c r="E8" s="414" t="inlineStr">
+      <c r="E8" s="415" t="inlineStr">
         <is>
           <t>Hojas de boldo</t>
         </is>
       </c>
-      <c r="F8" s="418" t="n">
+      <c r="F8" s="419" t="n">
         <v>400</v>
       </c>
-      <c r="G8" s="418" t="n">
+      <c r="G8" s="419" t="n">
         <v>1250</v>
       </c>
       <c r="H8" s="47">
@@ -12013,31 +12014,31 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="414" t="n">
+      <c r="A9" s="415" t="n">
         <v>205</v>
       </c>
-      <c r="B9" s="417" t="n">
+      <c r="B9" s="418" t="n">
         <v>46321</v>
       </c>
-      <c r="C9" s="414" t="inlineStr">
+      <c r="C9" s="415" t="inlineStr">
         <is>
           <t>Luis Araya (recolector)</t>
         </is>
       </c>
-      <c r="D9" s="414" t="inlineStr">
+      <c r="D9" s="415" t="inlineStr">
         <is>
           <t>15.555.555-6</t>
         </is>
       </c>
-      <c r="E9" s="414" t="inlineStr">
+      <c r="E9" s="415" t="inlineStr">
         <is>
           <t>Frutos de espino</t>
         </is>
       </c>
-      <c r="F9" s="418" t="n">
+      <c r="F9" s="419" t="n">
         <v>900</v>
       </c>
-      <c r="G9" s="418" t="n">
+      <c r="G9" s="419" t="n">
         <v>1500</v>
       </c>
       <c r="H9" s="47">
@@ -12099,7 +12100,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G46"/>
+  <dimension ref="A1:G40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -12112,32 +12113,32 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="419" t="inlineStr">
+      <c r="A1" s="420" t="inlineStr">
         <is>
           <t>Asiento</t>
         </is>
       </c>
-      <c r="B1" s="419" t="inlineStr">
+      <c r="B1" s="420" t="inlineStr">
         <is>
           <t>Fecha</t>
         </is>
       </c>
-      <c r="C1" s="419" t="inlineStr">
+      <c r="C1" s="420" t="inlineStr">
         <is>
           <t>Cuenta</t>
         </is>
       </c>
-      <c r="D1" s="419" t="inlineStr">
+      <c r="D1" s="420" t="inlineStr">
         <is>
           <t>Glosa</t>
         </is>
       </c>
-      <c r="E1" s="419" t="inlineStr">
+      <c r="E1" s="420" t="inlineStr">
         <is>
           <t>Debe</t>
         </is>
       </c>
-      <c r="F1" s="419" t="inlineStr">
+      <c r="F1" s="420" t="inlineStr">
         <is>
           <t>Haber</t>
         </is>
@@ -12147,7 +12148,7 @@
       <c r="A2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="420" t="n">
+      <c r="B2" s="421" t="n">
         <v>46297</v>
       </c>
       <c r="C2" t="inlineStr">
@@ -12161,7 +12162,7 @@
         </is>
       </c>
       <c r="E2" s="47">
-        <f>'L. COMPRAS'!H7</f>
+        <f>'L. COMPRAS'!H7+'L. COMPRAS'!I7</f>
         <v/>
       </c>
     </row>
@@ -12169,12 +12170,12 @@
       <c r="A3" t="n">
         <v>1</v>
       </c>
-      <c r="B3" s="420" t="n">
+      <c r="B3" s="421" t="n">
         <v>46297</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>1.1.04 IVA crédito fiscal</t>
+          <t>2.1.01 Proveedores</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -12182,8 +12183,8 @@
           <t>Factura de compra N°201: Rosa mosqueta (IVA retenido)</t>
         </is>
       </c>
-      <c r="E3" s="47">
-        <f>'L. COMPRAS'!I7</f>
+      <c r="F3" s="47">
+        <f>'L. COMPRAS'!J7-'L. COMPRAS'!K7</f>
         <v/>
       </c>
     </row>
@@ -12191,12 +12192,12 @@
       <c r="A4" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="420" t="n">
+      <c r="B4" s="421" t="n">
         <v>46297</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2.1.01 Proveedores</t>
+          <t>2.1.09 IVA retenido por pagar</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -12205,29 +12206,29 @@
         </is>
       </c>
       <c r="F4" s="47">
-        <f>'L. COMPRAS'!J7-'L. COMPRAS'!K7</f>
+        <f>'L. COMPRAS'!K7</f>
         <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>1</v>
-      </c>
-      <c r="B5" s="420" t="n">
-        <v>46297</v>
+        <v>2</v>
+      </c>
+      <c r="B5" s="421" t="n">
+        <v>46301</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2.1.09 IVA retenido por pagar</t>
+          <t>1.1.13 Inventario mercaderías</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Factura de compra N°201: Rosa mosqueta (IVA retenido)</t>
-        </is>
-      </c>
-      <c r="F5" s="47">
-        <f>'L. COMPRAS'!K7</f>
+          <t>Factura de compra N°202: Hongos (IVA retenido)</t>
+        </is>
+      </c>
+      <c r="E5" s="47">
+        <f>'L. COMPRAS'!H8+'L. COMPRAS'!I8</f>
         <v/>
       </c>
     </row>
@@ -12235,12 +12236,12 @@
       <c r="A6" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="420" t="n">
+      <c r="B6" s="421" t="n">
         <v>46301</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>1.1.13 Inventario mercaderías</t>
+          <t>2.1.01 Proveedores</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -12248,8 +12249,8 @@
           <t>Factura de compra N°202: Hongos (IVA retenido)</t>
         </is>
       </c>
-      <c r="E6" s="47">
-        <f>'L. COMPRAS'!H8</f>
+      <c r="F6" s="47">
+        <f>'L. COMPRAS'!J8-'L. COMPRAS'!K8</f>
         <v/>
       </c>
     </row>
@@ -12257,12 +12258,12 @@
       <c r="A7" t="n">
         <v>2</v>
       </c>
-      <c r="B7" s="420" t="n">
+      <c r="B7" s="421" t="n">
         <v>46301</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>1.1.04 IVA crédito fiscal</t>
+          <t>2.1.09 IVA retenido por pagar</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -12270,52 +12271,52 @@
           <t>Factura de compra N°202: Hongos (IVA retenido)</t>
         </is>
       </c>
-      <c r="E7" s="47">
-        <f>'L. COMPRAS'!I8</f>
+      <c r="F7" s="47">
+        <f>'L. COMPRAS'!K8</f>
         <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>2</v>
-      </c>
-      <c r="B8" s="420" t="n">
-        <v>46301</v>
+        <v>3</v>
+      </c>
+      <c r="B8" s="421" t="n">
+        <v>46307</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2.1.01 Proveedores</t>
+          <t>1.1.13 Inventario mercaderías</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Factura de compra N°202: Hongos (IVA retenido)</t>
-        </is>
-      </c>
-      <c r="F8" s="47">
-        <f>'L. COMPRAS'!J8-'L. COMPRAS'!K8</f>
+          <t>Factura de compra N°203: Mora (IVA retenido)</t>
+        </is>
+      </c>
+      <c r="E8" s="47">
+        <f>'L. COMPRAS'!H9+'L. COMPRAS'!I9</f>
         <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>2</v>
-      </c>
-      <c r="B9" s="420" t="n">
-        <v>46301</v>
+        <v>3</v>
+      </c>
+      <c r="B9" s="421" t="n">
+        <v>46307</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2.1.09 IVA retenido por pagar</t>
+          <t>2.1.01 Proveedores</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Factura de compra N°202: Hongos (IVA retenido)</t>
+          <t>Factura de compra N°203: Mora (IVA retenido)</t>
         </is>
       </c>
       <c r="F9" s="47">
-        <f>'L. COMPRAS'!K8</f>
+        <f>'L. COMPRAS'!J9-'L. COMPRAS'!K9</f>
         <v/>
       </c>
     </row>
@@ -12323,12 +12324,12 @@
       <c r="A10" t="n">
         <v>3</v>
       </c>
-      <c r="B10" s="420" t="n">
+      <c r="B10" s="421" t="n">
         <v>46307</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>1.1.13 Inventario mercaderías</t>
+          <t>2.1.09 IVA retenido por pagar</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -12336,39 +12337,39 @@
           <t>Factura de compra N°203: Mora (IVA retenido)</t>
         </is>
       </c>
-      <c r="E10" s="47">
-        <f>'L. COMPRAS'!H9</f>
+      <c r="F10" s="47">
+        <f>'L. COMPRAS'!K9</f>
         <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>3</v>
-      </c>
-      <c r="B11" s="420" t="n">
-        <v>46307</v>
+        <v>4</v>
+      </c>
+      <c r="B11" s="421" t="n">
+        <v>46314</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1.1.04 IVA crédito fiscal</t>
+          <t>1.1.13 Inventario mercaderías</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Factura de compra N°203: Mora (IVA retenido)</t>
+          <t>Factura de compra N°204: Hojas de boldo (IVA retenido)</t>
         </is>
       </c>
       <c r="E11" s="47">
-        <f>'L. COMPRAS'!I9</f>
+        <f>'L. COMPRAS'!H10+'L. COMPRAS'!I10</f>
         <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>3</v>
-      </c>
-      <c r="B12" s="420" t="n">
-        <v>46307</v>
+        <v>4</v>
+      </c>
+      <c r="B12" s="421" t="n">
+        <v>46314</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -12377,20 +12378,20 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Factura de compra N°203: Mora (IVA retenido)</t>
+          <t>Factura de compra N°204: Hojas de boldo (IVA retenido)</t>
         </is>
       </c>
       <c r="F12" s="47">
-        <f>'L. COMPRAS'!J9-'L. COMPRAS'!K9</f>
+        <f>'L. COMPRAS'!J10-'L. COMPRAS'!K10</f>
         <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>3</v>
-      </c>
-      <c r="B13" s="420" t="n">
-        <v>46307</v>
+        <v>4</v>
+      </c>
+      <c r="B13" s="421" t="n">
+        <v>46314</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -12399,20 +12400,20 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Factura de compra N°203: Mora (IVA retenido)</t>
+          <t>Factura de compra N°204: Hojas de boldo (IVA retenido)</t>
         </is>
       </c>
       <c r="F13" s="47">
-        <f>'L. COMPRAS'!K9</f>
+        <f>'L. COMPRAS'!K10</f>
         <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>4</v>
-      </c>
-      <c r="B14" s="420" t="n">
-        <v>46314</v>
+        <v>5</v>
+      </c>
+      <c r="B14" s="421" t="n">
+        <v>46321</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -12421,482 +12422,482 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Factura de compra N°204: Hojas de boldo (IVA retenido)</t>
+          <t>Factura de compra N°205: Frutos de espino (IVA retenido)</t>
         </is>
       </c>
       <c r="E14" s="47">
-        <f>'L. COMPRAS'!H10</f>
+        <f>'L. COMPRAS'!H11+'L. COMPRAS'!I11</f>
         <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>4</v>
-      </c>
-      <c r="B15" s="420" t="n">
-        <v>46314</v>
+        <v>5</v>
+      </c>
+      <c r="B15" s="421" t="n">
+        <v>46321</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>1.1.04 IVA crédito fiscal</t>
+          <t>2.1.01 Proveedores</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Factura de compra N°204: Hojas de boldo (IVA retenido)</t>
-        </is>
-      </c>
-      <c r="E15" s="47">
-        <f>'L. COMPRAS'!I10</f>
+          <t>Factura de compra N°205: Frutos de espino (IVA retenido)</t>
+        </is>
+      </c>
+      <c r="F15" s="47">
+        <f>'L. COMPRAS'!J11-'L. COMPRAS'!K11</f>
         <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>4</v>
-      </c>
-      <c r="B16" s="420" t="n">
-        <v>46314</v>
+        <v>5</v>
+      </c>
+      <c r="B16" s="421" t="n">
+        <v>46321</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2.1.01 Proveedores</t>
+          <t>2.1.09 IVA retenido por pagar</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Factura de compra N°204: Hojas de boldo (IVA retenido)</t>
+          <t>Factura de compra N°205: Frutos de espino (IVA retenido)</t>
         </is>
       </c>
       <c r="F16" s="47">
-        <f>'L. COMPRAS'!J10-'L. COMPRAS'!K10</f>
+        <f>'L. COMPRAS'!K11</f>
         <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>4</v>
-      </c>
-      <c r="B17" s="420" t="n">
-        <v>46314</v>
+        <v>6</v>
+      </c>
+      <c r="B17" s="421" t="n">
+        <v>46300</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2.1.09 IVA retenido por pagar</t>
+          <t>1.1.03 Clientes</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Factura de compra N°204: Hojas de boldo (IVA retenido)</t>
-        </is>
-      </c>
-      <c r="F17" s="47">
-        <f>'L. COMPRAS'!K10</f>
+          <t>Factura de venta N°101 a Exportadora Andes SpA</t>
+        </is>
+      </c>
+      <c r="E17" s="47">
+        <f>'L. VENTAS'!J6</f>
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>5</v>
-      </c>
-      <c r="B18" s="420" t="n">
-        <v>46321</v>
+        <v>6</v>
+      </c>
+      <c r="B18" s="421" t="n">
+        <v>46300</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>1.1.13 Inventario mercaderías</t>
+          <t>4.1.01 Ventas</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Factura de compra N°205: Frutos de espino (IVA retenido)</t>
-        </is>
-      </c>
-      <c r="E18" s="47">
-        <f>'L. COMPRAS'!H11</f>
+          <t>Factura de venta N°101 a Exportadora Andes SpA</t>
+        </is>
+      </c>
+      <c r="F18" s="47">
+        <f>'L. VENTAS'!H6</f>
         <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>5</v>
-      </c>
-      <c r="B19" s="420" t="n">
-        <v>46321</v>
+        <v>6</v>
+      </c>
+      <c r="B19" s="421" t="n">
+        <v>46300</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>1.1.04 IVA crédito fiscal</t>
+          <t>2.1.02 IVA débito fiscal</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Factura de compra N°205: Frutos de espino (IVA retenido)</t>
-        </is>
-      </c>
-      <c r="E19" s="47">
-        <f>'L. COMPRAS'!I11</f>
+          <t>Factura de venta N°101 a Exportadora Andes SpA</t>
+        </is>
+      </c>
+      <c r="F19" s="47">
+        <f>'L. VENTAS'!I6</f>
         <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>5</v>
-      </c>
-      <c r="B20" s="420" t="n">
-        <v>46321</v>
+        <v>7</v>
+      </c>
+      <c r="B20" s="421" t="n">
+        <v>46304</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2.1.01 Proveedores</t>
+          <t>1.1.03 Clientes</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Factura de compra N°205: Frutos de espino (IVA retenido)</t>
-        </is>
-      </c>
-      <c r="F20" s="47">
-        <f>'L. COMPRAS'!J11-'L. COMPRAS'!K11</f>
+          <t>Factura de venta N°102 a Agroindustrial Sur Ltda.</t>
+        </is>
+      </c>
+      <c r="E20" s="47">
+        <f>'L. VENTAS'!J7</f>
         <v/>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>5</v>
-      </c>
-      <c r="B21" s="420" t="n">
-        <v>46321</v>
+        <v>7</v>
+      </c>
+      <c r="B21" s="421" t="n">
+        <v>46304</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2.1.09 IVA retenido por pagar</t>
+          <t>4.1.01 Ventas</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Factura de compra N°205: Frutos de espino (IVA retenido)</t>
+          <t>Factura de venta N°102 a Agroindustrial Sur Ltda.</t>
         </is>
       </c>
       <c r="F21" s="47">
-        <f>'L. COMPRAS'!K11</f>
+        <f>'L. VENTAS'!H7</f>
         <v/>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>6</v>
-      </c>
-      <c r="B22" s="420" t="n">
-        <v>46300</v>
+        <v>7</v>
+      </c>
+      <c r="B22" s="421" t="n">
+        <v>46304</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>1.1.03 Clientes</t>
+          <t>2.1.02 IVA débito fiscal</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Factura de venta N°101 a Exportadora Andes SpA</t>
-        </is>
-      </c>
-      <c r="E22" s="47">
-        <f>'L. VENTAS'!J6</f>
+          <t>Factura de venta N°102 a Agroindustrial Sur Ltda.</t>
+        </is>
+      </c>
+      <c r="F22" s="47">
+        <f>'L. VENTAS'!I7</f>
         <v/>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>6</v>
-      </c>
-      <c r="B23" s="420" t="n">
-        <v>46300</v>
+        <v>8</v>
+      </c>
+      <c r="B23" s="421" t="n">
+        <v>46309</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>4.1.01 Ventas</t>
+          <t>1.1.03 Clientes</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Factura de venta N°101 a Exportadora Andes SpA</t>
-        </is>
-      </c>
-      <c r="F23" s="47">
-        <f>'L. VENTAS'!H6</f>
+          <t>Factura de venta N°103 a Hierbas del Valle S.A.</t>
+        </is>
+      </c>
+      <c r="E23" s="47">
+        <f>'L. VENTAS'!J8</f>
         <v/>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>6</v>
-      </c>
-      <c r="B24" s="420" t="n">
-        <v>46300</v>
+        <v>8</v>
+      </c>
+      <c r="B24" s="421" t="n">
+        <v>46309</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2.1.02 IVA débito fiscal</t>
+          <t>4.1.01 Ventas</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Factura de venta N°101 a Exportadora Andes SpA</t>
+          <t>Factura de venta N°103 a Hierbas del Valle S.A.</t>
         </is>
       </c>
       <c r="F24" s="47">
-        <f>'L. VENTAS'!I6</f>
+        <f>'L. VENTAS'!H8</f>
         <v/>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>7</v>
-      </c>
-      <c r="B25" s="420" t="n">
-        <v>46304</v>
+        <v>8</v>
+      </c>
+      <c r="B25" s="421" t="n">
+        <v>46309</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>1.1.03 Clientes</t>
+          <t>2.1.02 IVA débito fiscal</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Factura de venta N°102 a Agroindustrial Sur Ltda.</t>
-        </is>
-      </c>
-      <c r="E25" s="47">
-        <f>'L. VENTAS'!J7</f>
+          <t>Factura de venta N°103 a Hierbas del Valle S.A.</t>
+        </is>
+      </c>
+      <c r="F25" s="47">
+        <f>'L. VENTAS'!I8</f>
         <v/>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>7</v>
-      </c>
-      <c r="B26" s="420" t="n">
-        <v>46304</v>
+        <v>9</v>
+      </c>
+      <c r="B26" s="421" t="n">
+        <v>46316</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>4.1.01 Ventas</t>
+          <t>1.1.03 Clientes</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Factura de venta N°102 a Agroindustrial Sur Ltda.</t>
-        </is>
-      </c>
-      <c r="F26" s="47">
-        <f>'L. VENTAS'!H7</f>
+          <t>Factura de venta N°104 a Comercial Maule SpA</t>
+        </is>
+      </c>
+      <c r="E26" s="47">
+        <f>'L. VENTAS'!J9</f>
         <v/>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>7</v>
-      </c>
-      <c r="B27" s="420" t="n">
-        <v>46304</v>
+        <v>9</v>
+      </c>
+      <c r="B27" s="421" t="n">
+        <v>46316</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2.1.02 IVA débito fiscal</t>
+          <t>4.1.01 Ventas</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Factura de venta N°102 a Agroindustrial Sur Ltda.</t>
+          <t>Factura de venta N°104 a Comercial Maule SpA</t>
         </is>
       </c>
       <c r="F27" s="47">
-        <f>'L. VENTAS'!I7</f>
+        <f>'L. VENTAS'!H9</f>
         <v/>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>8</v>
-      </c>
-      <c r="B28" s="420" t="n">
-        <v>46309</v>
+        <v>9</v>
+      </c>
+      <c r="B28" s="421" t="n">
+        <v>46316</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>1.1.03 Clientes</t>
+          <t>2.1.02 IVA débito fiscal</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Factura de venta N°103 a Hierbas del Valle S.A.</t>
-        </is>
-      </c>
-      <c r="E28" s="47">
-        <f>'L. VENTAS'!J8</f>
+          <t>Factura de venta N°104 a Comercial Maule SpA</t>
+        </is>
+      </c>
+      <c r="F28" s="47">
+        <f>'L. VENTAS'!I9</f>
         <v/>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>8</v>
-      </c>
-      <c r="B29" s="420" t="n">
-        <v>46309</v>
+        <v>10</v>
+      </c>
+      <c r="B29" s="421" t="n">
+        <v>46323</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>4.1.01 Ventas</t>
+          <t>1.1.03 Clientes</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Factura de venta N°103 a Hierbas del Valle S.A.</t>
-        </is>
-      </c>
-      <c r="F29" s="47">
-        <f>'L. VENTAS'!H8</f>
+          <t>Factura de venta N°105 a Distribuidora Bío Bío Ltda.</t>
+        </is>
+      </c>
+      <c r="E29" s="47">
+        <f>'L. VENTAS'!J10</f>
         <v/>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>8</v>
-      </c>
-      <c r="B30" s="420" t="n">
-        <v>46309</v>
+        <v>10</v>
+      </c>
+      <c r="B30" s="421" t="n">
+        <v>46323</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2.1.02 IVA débito fiscal</t>
+          <t>4.1.01 Ventas</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Factura de venta N°103 a Hierbas del Valle S.A.</t>
+          <t>Factura de venta N°105 a Distribuidora Bío Bío Ltda.</t>
         </is>
       </c>
       <c r="F30" s="47">
-        <f>'L. VENTAS'!I8</f>
+        <f>'L. VENTAS'!H10</f>
         <v/>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>9</v>
-      </c>
-      <c r="B31" s="420" t="n">
-        <v>46316</v>
+        <v>10</v>
+      </c>
+      <c r="B31" s="421" t="n">
+        <v>46323</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>1.1.03 Clientes</t>
+          <t>2.1.02 IVA débito fiscal</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Factura de venta N°104 a Comercial Maule SpA</t>
-        </is>
-      </c>
-      <c r="E31" s="47">
-        <f>'L. VENTAS'!J9</f>
+          <t>Factura de venta N°105 a Distribuidora Bío Bío Ltda.</t>
+        </is>
+      </c>
+      <c r="F31" s="47">
+        <f>'L. VENTAS'!I10</f>
         <v/>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>9</v>
-      </c>
-      <c r="B32" s="420" t="n">
-        <v>46316</v>
+        <v>11</v>
+      </c>
+      <c r="B32" s="421" t="n">
+        <v>46326</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>4.1.01 Ventas</t>
+          <t>5.1.01 Costo de ventas</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Factura de venta N°104 a Comercial Maule SpA</t>
-        </is>
-      </c>
-      <c r="F32" s="47">
-        <f>'L. VENTAS'!H9</f>
+          <t>Costo de las ventas del mes</t>
+        </is>
+      </c>
+      <c r="E32" s="47">
+        <f>'L. VENTAS'!P19</f>
         <v/>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>9</v>
-      </c>
-      <c r="B33" s="420" t="n">
-        <v>46316</v>
+        <v>11</v>
+      </c>
+      <c r="B33" s="421" t="n">
+        <v>46326</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>2.1.02 IVA débito fiscal</t>
+          <t>1.1.13 Inventario mercaderías</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Factura de venta N°104 a Comercial Maule SpA</t>
+          <t>Costo de las ventas del mes</t>
         </is>
       </c>
       <c r="F33" s="47">
-        <f>'L. VENTAS'!I9</f>
+        <f>'L. VENTAS'!P19</f>
         <v/>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>10</v>
-      </c>
-      <c r="B34" s="420" t="n">
-        <v>46323</v>
+        <v>12</v>
+      </c>
+      <c r="B34" s="421" t="n">
+        <v>46326</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>1.1.03 Clientes</t>
+          <t>2.1.01 Proveedores</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Factura de venta N°105 a Distribuidora Bío Bío Ltda.</t>
+          <t>Pago a los proveedores</t>
         </is>
       </c>
       <c r="E34" s="47">
-        <f>'L. VENTAS'!J10</f>
+        <f>'L. COMPRAS'!O16</f>
         <v/>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>10</v>
-      </c>
-      <c r="B35" s="420" t="n">
-        <v>46323</v>
+        <v>12</v>
+      </c>
+      <c r="B35" s="421" t="n">
+        <v>46326</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>4.1.01 Ventas</t>
+          <t>1.1.02 Banco</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Factura de venta N°105 a Distribuidora Bío Bío Ltda.</t>
+          <t>Pago a los proveedores</t>
         </is>
       </c>
       <c r="F35" s="47">
-        <f>'L. VENTAS'!H10</f>
+        <f>'L. COMPRAS'!O16</f>
         <v/>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>10</v>
-      </c>
-      <c r="B36" s="420" t="n">
-        <v>46323</v>
+        <v>13</v>
+      </c>
+      <c r="B36" s="421" t="n">
+        <v>46338</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -12905,228 +12906,96 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Factura de venta N°105 a Distribuidora Bío Bío Ltda.</t>
-        </is>
-      </c>
-      <c r="F36" s="47">
-        <f>'L. VENTAS'!I10</f>
+          <t>F29: débito, IVA retenido y PPM</t>
+        </is>
+      </c>
+      <c r="E36" s="47">
+        <f>'FORMULARIO 29'!AP16</f>
         <v/>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>11</v>
-      </c>
-      <c r="B37" s="420" t="n">
-        <v>46326</v>
+        <v>13</v>
+      </c>
+      <c r="B37" s="421" t="n">
+        <v>46338</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>5.1.01 Costo de ventas</t>
+          <t>2.1.09 IVA retenido por pagar</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Costo de las ventas del mes</t>
+          <t>F29: débito, IVA retenido y PPM</t>
         </is>
       </c>
       <c r="E37" s="47">
-        <f>'L. VENTAS'!P19</f>
+        <f>'FORMULARIO 29'!AP97</f>
         <v/>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>11</v>
-      </c>
-      <c r="B38" s="420" t="n">
-        <v>46326</v>
+        <v>13</v>
+      </c>
+      <c r="B38" s="421" t="n">
+        <v>46338</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>1.1.13 Inventario mercaderías</t>
+          <t>1.1.05 PPM por recuperar</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Costo de las ventas del mes</t>
-        </is>
-      </c>
-      <c r="F38" s="47">
-        <f>'L. VENTAS'!P19</f>
+          <t>F29: débito, IVA retenido y PPM</t>
+        </is>
+      </c>
+      <c r="E38" s="47">
+        <f>'FORMULARIO 29'!AP74</f>
         <v/>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>12</v>
-      </c>
-      <c r="B39" s="420" t="n">
-        <v>46326</v>
+        <v>13</v>
+      </c>
+      <c r="B39" s="421" t="n">
+        <v>46338</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>2.1.01 Proveedores</t>
+          <t>1.1.02 Banco</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Pago a los proveedores</t>
-        </is>
-      </c>
-      <c r="E39" s="47">
-        <f>'L. COMPRAS'!O16</f>
+          <t>F29: débito, IVA retenido y PPM</t>
+        </is>
+      </c>
+      <c r="F39" s="47">
+        <f>'FORMULARIO 29'!AP92</f>
         <v/>
       </c>
     </row>
     <row r="40">
-      <c r="A40" t="n">
-        <v>12</v>
-      </c>
-      <c r="B40" s="420" t="n">
-        <v>46326</v>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>1.1.02 Banco</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>Pago a los proveedores</t>
-        </is>
+      <c r="D40" s="336" t="inlineStr">
+        <is>
+          <t>SUMAS IGUALES</t>
+        </is>
+      </c>
+      <c r="E40" s="47">
+        <f>SUM(E2:E39)</f>
+        <v/>
       </c>
       <c r="F40" s="47">
-        <f>'L. COMPRAS'!O16</f>
-        <v/>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="n">
-        <v>13</v>
-      </c>
-      <c r="B41" s="420" t="n">
-        <v>46338</v>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>2.1.02 IVA débito fiscal</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>F29: débito, IVA retenido, crédito y PPM</t>
-        </is>
-      </c>
-      <c r="E41" s="47">
-        <f>'FORMULARIO 29'!AP16</f>
-        <v/>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="n">
-        <v>13</v>
-      </c>
-      <c r="B42" s="420" t="n">
-        <v>46338</v>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>2.1.09 IVA retenido por pagar</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>F29: débito, IVA retenido, crédito y PPM</t>
-        </is>
-      </c>
-      <c r="E42" s="47">
-        <f>'FORMULARIO 29'!AP97</f>
-        <v/>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="n">
-        <v>13</v>
-      </c>
-      <c r="B43" s="420" t="n">
-        <v>46338</v>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>1.1.05 PPM por recuperar</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>F29: débito, IVA retenido, crédito y PPM</t>
-        </is>
-      </c>
-      <c r="E43" s="47">
-        <f>'FORMULARIO 29'!AP74</f>
-        <v/>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="n">
-        <v>13</v>
-      </c>
-      <c r="B44" s="420" t="n">
-        <v>46338</v>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>1.1.04 IVA crédito fiscal</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>F29: débito, IVA retenido, crédito y PPM</t>
-        </is>
-      </c>
-      <c r="F44" s="47">
-        <f>'FORMULARIO 29'!AP38</f>
-        <v/>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="n">
-        <v>13</v>
-      </c>
-      <c r="B45" s="420" t="n">
-        <v>46338</v>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>1.1.02 Banco</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>F29: débito, IVA retenido, crédito y PPM</t>
-        </is>
-      </c>
-      <c r="F45" s="47">
-        <f>'FORMULARIO 29'!AP92</f>
-        <v/>
-      </c>
-    </row>
-    <row r="46">
-      <c r="D46" s="336" t="inlineStr">
-        <is>
-          <t>SUMAS IGUALES</t>
-        </is>
-      </c>
-      <c r="E46" s="47">
-        <f>SUM(E2:E45)</f>
-        <v/>
-      </c>
-      <c r="F46" s="47">
-        <f>SUM(F2:F45)</f>
-        <v/>
-      </c>
-      <c r="G46">
-        <f>IF(E46=F46,"Cuadra","NO CUADRA")</f>
+        <f>SUM(F2:F39)</f>
+        <v/>
+      </c>
+      <c r="G40">
+        <f>IF(E40=F40,"Cuadra","NO CUADRA")</f>
         <v/>
       </c>
     </row>
@@ -13170,47 +13039,47 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="416" t="inlineStr">
+      <c r="A4" s="417" t="inlineStr">
         <is>
           <t>RUT del vendedor (retenido)</t>
         </is>
       </c>
-      <c r="B4" s="416" t="inlineStr">
+      <c r="B4" s="417" t="inlineStr">
         <is>
           <t>Código de producto (F3500)</t>
         </is>
       </c>
-      <c r="C4" s="416" t="inlineStr">
+      <c r="C4" s="417" t="inlineStr">
         <is>
           <t>Producto</t>
         </is>
       </c>
-      <c r="D4" s="416" t="inlineStr">
+      <c r="D4" s="417" t="inlineStr">
         <is>
           <t>Tipo de documento</t>
         </is>
       </c>
-      <c r="E4" s="416" t="inlineStr">
+      <c r="E4" s="417" t="inlineStr">
         <is>
           <t>N° documento</t>
         </is>
       </c>
-      <c r="F4" s="416" t="inlineStr">
+      <c r="F4" s="417" t="inlineStr">
         <is>
           <t>Fecha</t>
         </is>
       </c>
-      <c r="G4" s="416" t="inlineStr">
+      <c r="G4" s="417" t="inlineStr">
         <is>
           <t>Cantidad</t>
         </is>
       </c>
-      <c r="H4" s="416" t="inlineStr">
+      <c r="H4" s="417" t="inlineStr">
         <is>
           <t>Unidad de medida (cód. 1)</t>
         </is>
       </c>
-      <c r="I4" s="416" t="inlineStr">
+      <c r="I4" s="417" t="inlineStr">
         <is>
           <t>IVA retenido total</t>
         </is>
@@ -13238,7 +13107,7 @@
         <f>'L. COMPRAS'!B7</f>
         <v/>
       </c>
-      <c r="F5" s="420">
+      <c r="F5" s="421">
         <f>'L. COMPRAS'!A7</f>
         <v/>
       </c>
@@ -13276,7 +13145,7 @@
         <f>'L. COMPRAS'!B8</f>
         <v/>
       </c>
-      <c r="F6" s="420">
+      <c r="F6" s="421">
         <f>'L. COMPRAS'!A8</f>
         <v/>
       </c>
@@ -13314,7 +13183,7 @@
         <f>'L. COMPRAS'!B9</f>
         <v/>
       </c>
-      <c r="F7" s="420">
+      <c r="F7" s="421">
         <f>'L. COMPRAS'!A9</f>
         <v/>
       </c>
@@ -13352,7 +13221,7 @@
         <f>'L. COMPRAS'!B10</f>
         <v/>
       </c>
-      <c r="F8" s="420">
+      <c r="F8" s="421">
         <f>'L. COMPRAS'!A10</f>
         <v/>
       </c>
@@ -13390,7 +13259,7 @@
         <f>'L. COMPRAS'!B11</f>
         <v/>
       </c>
-      <c r="F9" s="420">
+      <c r="F9" s="421">
         <f>'L. COMPRAS'!A11</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Trabajo Juan Castillo: verificado en sii.cl (Res. 4095, F29, F3500, código 31)
- El IVA de la factura de compra sí es crédito fiscal (Res. 4095 N° 6): F29 línea 25 (519/520), total 1.400.000
- Libro de compras con código 31 (IVA retenido silvestres)
- Texto oficial de la resolución en el Word; logo opcional desde base/logo.png
- Fuentes oficiales en docs/normativa/fuentes/; guía Claude in Chrome

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/trabajo_juan_castillo/cambio_sujeto_silvestres.xlsx
+++ b/trabajo_juan_castillo/cambio_sujeto_silvestres.xlsx
@@ -617,7 +617,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="171" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="422">
+  <cellXfs count="421">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1835,11 +1835,8 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="10" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="1">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="10" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-      <protection locked="1" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="14" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="1" hidden="1"/>
     </xf>
     <xf numFmtId="3" fontId="9" fillId="5" borderId="10" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="1">
@@ -2519,7 +2516,7 @@
       </c>
       <c r="K5" s="316" t="inlineStr">
         <is>
-          <t>IVA RETENIDO TOTAL (cód. 15)</t>
+          <t>IVA RETENIDO TOTAL (cód. 31 silvestres)</t>
         </is>
       </c>
       <c r="L5" s="100" t="inlineStr">
@@ -2783,7 +2780,7 @@
       </c>
       <c r="M11" s="6" t="n"/>
       <c r="N11" s="31">
-        <f>O5+K31</f>
+        <f>O5</f>
         <v/>
       </c>
       <c r="O11" s="1" t="n"/>
@@ -2874,8 +2871,9 @@
         </is>
       </c>
       <c r="M15" s="6" t="n"/>
-      <c r="N15" s="31" t="n">
-        <v>0</v>
+      <c r="N15" s="31">
+        <f>I31</f>
+        <v/>
       </c>
       <c r="O15" s="1" t="n"/>
     </row>
@@ -3508,7 +3506,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Las facturas de compra (DTE 46) las emite el comprador; el IVA retenido total no da derecho a crédito fiscal y se paga en el F29 (reverso, código 39).</t>
+          <t>Las facturas de compra (DTE 46) las emite el comprador; su IVA es crédito fiscal (Res. 4095, N° 6) y el IVA retenido se paga en el F29 (reverso, código 39). Código 31 = IVA retenido silvestres (se informa como retención total).</t>
         </is>
       </c>
       <c r="F66" s="98" t="n"/>
@@ -4636,8 +4634,9 @@
         <v/>
       </c>
       <c r="C75" s="6" t="n"/>
-      <c r="D75" s="38" t="n">
-        <v>0</v>
+      <c r="D75" s="38">
+        <f>'L. COMPRAS'!I64</f>
+        <v/>
       </c>
       <c r="E75" s="6" t="n"/>
       <c r="G75" s="325" t="inlineStr">
@@ -7298,68 +7297,62 @@
       <c r="A34" s="8" t="n"/>
       <c r="B34" s="351" t="n"/>
       <c r="C34" s="352" t="n"/>
-      <c r="D34" s="356" t="n">
+      <c r="D34" s="146" t="n">
         <v>22</v>
       </c>
-      <c r="E34" s="357" t="n"/>
-      <c r="F34" s="376" t="inlineStr">
+      <c r="E34" s="355" t="n"/>
+      <c r="F34" s="204" t="inlineStr">
         <is>
           <t>Sin Derecho a Credito Fiscal</t>
         </is>
       </c>
-      <c r="G34" s="377" t="n"/>
-      <c r="H34" s="358" t="inlineStr">
+      <c r="G34" s="342" t="n"/>
+      <c r="H34" s="152" t="inlineStr">
         <is>
           <t>Internas afectas</t>
         </is>
       </c>
-      <c r="I34" s="359" t="n"/>
-      <c r="J34" s="359" t="n"/>
-      <c r="K34" s="359" t="n"/>
-      <c r="L34" s="359" t="n"/>
-      <c r="M34" s="359" t="n"/>
-      <c r="N34" s="359" t="n"/>
-      <c r="O34" s="359" t="n"/>
-      <c r="P34" s="359" t="n"/>
-      <c r="Q34" s="359" t="n"/>
-      <c r="R34" s="359" t="n"/>
-      <c r="S34" s="359" t="n"/>
-      <c r="T34" s="359" t="n"/>
-      <c r="U34" s="359" t="n"/>
-      <c r="V34" s="360" t="n"/>
-      <c r="W34" s="361" t="n">
+      <c r="I34" s="339" t="n"/>
+      <c r="J34" s="339" t="n"/>
+      <c r="K34" s="339" t="n"/>
+      <c r="L34" s="339" t="n"/>
+      <c r="M34" s="339" t="n"/>
+      <c r="N34" s="339" t="n"/>
+      <c r="O34" s="339" t="n"/>
+      <c r="P34" s="339" t="n"/>
+      <c r="Q34" s="339" t="n"/>
+      <c r="R34" s="339" t="n"/>
+      <c r="S34" s="339" t="n"/>
+      <c r="T34" s="339" t="n"/>
+      <c r="U34" s="339" t="n"/>
+      <c r="V34" s="340" t="n"/>
+      <c r="W34" s="153" t="n">
         <v>564</v>
       </c>
-      <c r="X34" s="360" t="n"/>
-      <c r="Y34" s="371">
-        <f>COUNT('L. COMPRAS'!B7:B30)</f>
-        <v/>
-      </c>
-      <c r="Z34" s="363" t="n"/>
-      <c r="AA34" s="363" t="n"/>
-      <c r="AB34" s="363" t="n"/>
-      <c r="AC34" s="363" t="n"/>
-      <c r="AD34" s="363" t="n"/>
-      <c r="AE34" s="363" t="n"/>
-      <c r="AF34" s="363" t="n"/>
-      <c r="AG34" s="363" t="n"/>
-      <c r="AH34" s="363" t="n"/>
-      <c r="AI34" s="363" t="n"/>
-      <c r="AJ34" s="363" t="n"/>
-      <c r="AK34" s="363" t="n"/>
-      <c r="AL34" s="363" t="n"/>
-      <c r="AM34" s="364" t="n"/>
-      <c r="AN34" s="356" t="n">
+      <c r="X34" s="340" t="n"/>
+      <c r="Y34" s="369" t="n"/>
+      <c r="Z34" s="349" t="n"/>
+      <c r="AA34" s="349" t="n"/>
+      <c r="AB34" s="349" t="n"/>
+      <c r="AC34" s="349" t="n"/>
+      <c r="AD34" s="349" t="n"/>
+      <c r="AE34" s="349" t="n"/>
+      <c r="AF34" s="349" t="n"/>
+      <c r="AG34" s="349" t="n"/>
+      <c r="AH34" s="349" t="n"/>
+      <c r="AI34" s="349" t="n"/>
+      <c r="AJ34" s="349" t="n"/>
+      <c r="AK34" s="349" t="n"/>
+      <c r="AL34" s="349" t="n"/>
+      <c r="AM34" s="350" t="n"/>
+      <c r="AN34" s="155" t="n">
         <v>521</v>
       </c>
-      <c r="AO34" s="360" t="n"/>
-      <c r="AP34" s="378">
-        <f>'L. COMPRAS'!H31</f>
-        <v/>
-      </c>
-      <c r="AQ34" s="363" t="n"/>
-      <c r="AR34" s="364" t="n"/>
-      <c r="AS34" s="356" t="n"/>
+      <c r="AO34" s="340" t="n"/>
+      <c r="AP34" s="353" t="n"/>
+      <c r="AQ34" s="349" t="n"/>
+      <c r="AR34" s="350" t="n"/>
+      <c r="AS34" s="146" t="n"/>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="8" t="n"/>
@@ -7534,66 +7527,72 @@
       <c r="A38" s="8" t="n"/>
       <c r="B38" s="351" t="n"/>
       <c r="C38" s="352" t="n"/>
-      <c r="D38" s="146" t="n">
+      <c r="D38" s="356" t="n">
         <v>25</v>
       </c>
-      <c r="E38" s="355" t="n"/>
-      <c r="F38" s="209" t="inlineStr">
+      <c r="E38" s="357" t="n"/>
+      <c r="F38" s="376" t="inlineStr">
         <is>
           <t>Con Derecho a Crédito Fiscal</t>
         </is>
       </c>
-      <c r="G38" s="209" t="inlineStr">
+      <c r="G38" s="376" t="inlineStr">
         <is>
           <t>Internas</t>
         </is>
       </c>
-      <c r="H38" s="152" t="inlineStr">
+      <c r="H38" s="358" t="inlineStr">
         <is>
           <t>Facturas recibidas del giro y Facturas de compra emitidas</t>
         </is>
       </c>
-      <c r="I38" s="339" t="n"/>
-      <c r="J38" s="339" t="n"/>
-      <c r="K38" s="339" t="n"/>
-      <c r="L38" s="339" t="n"/>
-      <c r="M38" s="339" t="n"/>
-      <c r="N38" s="339" t="n"/>
-      <c r="O38" s="339" t="n"/>
-      <c r="P38" s="339" t="n"/>
-      <c r="Q38" s="339" t="n"/>
-      <c r="R38" s="339" t="n"/>
-      <c r="S38" s="339" t="n"/>
-      <c r="T38" s="339" t="n"/>
-      <c r="U38" s="339" t="n"/>
-      <c r="V38" s="340" t="n"/>
-      <c r="W38" s="153" t="n">
+      <c r="I38" s="359" t="n"/>
+      <c r="J38" s="359" t="n"/>
+      <c r="K38" s="359" t="n"/>
+      <c r="L38" s="359" t="n"/>
+      <c r="M38" s="359" t="n"/>
+      <c r="N38" s="359" t="n"/>
+      <c r="O38" s="359" t="n"/>
+      <c r="P38" s="359" t="n"/>
+      <c r="Q38" s="359" t="n"/>
+      <c r="R38" s="359" t="n"/>
+      <c r="S38" s="359" t="n"/>
+      <c r="T38" s="359" t="n"/>
+      <c r="U38" s="359" t="n"/>
+      <c r="V38" s="360" t="n"/>
+      <c r="W38" s="361" t="n">
         <v>519</v>
       </c>
-      <c r="X38" s="340" t="n"/>
-      <c r="Y38" s="369" t="n"/>
-      <c r="Z38" s="349" t="n"/>
-      <c r="AA38" s="349" t="n"/>
-      <c r="AB38" s="349" t="n"/>
-      <c r="AC38" s="349" t="n"/>
-      <c r="AD38" s="349" t="n"/>
-      <c r="AE38" s="349" t="n"/>
-      <c r="AF38" s="349" t="n"/>
-      <c r="AG38" s="349" t="n"/>
-      <c r="AH38" s="349" t="n"/>
-      <c r="AI38" s="349" t="n"/>
-      <c r="AJ38" s="349" t="n"/>
-      <c r="AK38" s="349" t="n"/>
-      <c r="AL38" s="349" t="n"/>
-      <c r="AM38" s="350" t="n"/>
-      <c r="AN38" s="155" t="n">
+      <c r="X38" s="360" t="n"/>
+      <c r="Y38" s="371">
+        <f>COUNT('L. COMPRAS'!B7:B30)</f>
+        <v/>
+      </c>
+      <c r="Z38" s="363" t="n"/>
+      <c r="AA38" s="363" t="n"/>
+      <c r="AB38" s="363" t="n"/>
+      <c r="AC38" s="363" t="n"/>
+      <c r="AD38" s="363" t="n"/>
+      <c r="AE38" s="363" t="n"/>
+      <c r="AF38" s="363" t="n"/>
+      <c r="AG38" s="363" t="n"/>
+      <c r="AH38" s="363" t="n"/>
+      <c r="AI38" s="363" t="n"/>
+      <c r="AJ38" s="363" t="n"/>
+      <c r="AK38" s="363" t="n"/>
+      <c r="AL38" s="363" t="n"/>
+      <c r="AM38" s="364" t="n"/>
+      <c r="AN38" s="356" t="n">
         <v>520</v>
       </c>
-      <c r="AO38" s="340" t="n"/>
-      <c r="AP38" s="353" t="n"/>
-      <c r="AQ38" s="349" t="n"/>
-      <c r="AR38" s="350" t="n"/>
-      <c r="AS38" s="89" t="inlineStr">
+      <c r="AO38" s="360" t="n"/>
+      <c r="AP38" s="377">
+        <f>'L. COMPRAS'!I31</f>
+        <v/>
+      </c>
+      <c r="AQ38" s="363" t="n"/>
+      <c r="AR38" s="364" t="n"/>
+      <c r="AS38" s="372" t="inlineStr">
         <is>
           <t>+</t>
         </is>
@@ -7609,7 +7608,7 @@
       <c r="E39" s="355" t="n"/>
       <c r="F39" s="355" t="n"/>
       <c r="G39" s="355" t="n"/>
-      <c r="H39" s="379" t="inlineStr">
+      <c r="H39" s="378" t="inlineStr">
         <is>
           <t>Facturas activo fijo</t>
         </is>
@@ -7632,7 +7631,7 @@
         <v>524</v>
       </c>
       <c r="X39" s="340" t="n"/>
-      <c r="Y39" s="380" t="n"/>
+      <c r="Y39" s="379" t="n"/>
       <c r="Z39" s="349" t="n"/>
       <c r="AA39" s="349" t="n"/>
       <c r="AB39" s="349" t="n"/>
@@ -7651,7 +7650,7 @@
         <v>525</v>
       </c>
       <c r="AO39" s="340" t="n"/>
-      <c r="AP39" s="381" t="n"/>
+      <c r="AP39" s="380" t="n"/>
       <c r="AQ39" s="349" t="n"/>
       <c r="AR39" s="350" t="n"/>
       <c r="AS39" s="89" t="inlineStr">
@@ -7731,7 +7730,7 @@
       <c r="E41" s="355" t="n"/>
       <c r="F41" s="355" t="n"/>
       <c r="G41" s="347" t="n"/>
-      <c r="H41" s="379" t="inlineStr">
+      <c r="H41" s="378" t="inlineStr">
         <is>
           <t>Notas de Débito recibidas</t>
         </is>
@@ -7754,7 +7753,7 @@
         <v>531</v>
       </c>
       <c r="X41" s="340" t="n"/>
-      <c r="Y41" s="380" t="n"/>
+      <c r="Y41" s="379" t="n"/>
       <c r="Z41" s="349" t="n"/>
       <c r="AA41" s="349" t="n"/>
       <c r="AB41" s="349" t="n"/>
@@ -7791,7 +7790,7 @@
       </c>
       <c r="E42" s="355" t="n"/>
       <c r="F42" s="355" t="n"/>
-      <c r="G42" s="382" t="inlineStr">
+      <c r="G42" s="381" t="inlineStr">
         <is>
           <t>Impor-tación</t>
         </is>
@@ -7915,7 +7914,7 @@
       <c r="D44" s="155" t="n">
         <v>31</v>
       </c>
-      <c r="E44" s="379" t="inlineStr">
+      <c r="E44" s="378" t="inlineStr">
         <is>
           <t>Remanente Crédito Fiscal del mes anterior</t>
         </is>
@@ -8334,29 +8333,29 @@
           <t>M3 Comprados con derecho a crédito</t>
         </is>
       </c>
-      <c r="S51" s="383" t="n"/>
-      <c r="T51" s="383" t="n"/>
-      <c r="U51" s="383" t="n"/>
-      <c r="V51" s="383" t="n"/>
-      <c r="W51" s="383" t="n"/>
-      <c r="X51" s="383" t="n"/>
-      <c r="Y51" s="383" t="n"/>
-      <c r="Z51" s="384" t="n"/>
+      <c r="S51" s="382" t="n"/>
+      <c r="T51" s="382" t="n"/>
+      <c r="U51" s="382" t="n"/>
+      <c r="V51" s="382" t="n"/>
+      <c r="W51" s="382" t="n"/>
+      <c r="X51" s="382" t="n"/>
+      <c r="Y51" s="382" t="n"/>
+      <c r="Z51" s="383" t="n"/>
       <c r="AC51" s="278" t="inlineStr">
         <is>
           <t>Componentes del Impuesto</t>
         </is>
       </c>
-      <c r="AD51" s="383" t="n"/>
-      <c r="AE51" s="383" t="n"/>
-      <c r="AF51" s="383" t="n"/>
-      <c r="AG51" s="383" t="n"/>
-      <c r="AH51" s="383" t="n"/>
-      <c r="AI51" s="383" t="n"/>
-      <c r="AJ51" s="383" t="n"/>
-      <c r="AK51" s="383" t="n"/>
-      <c r="AL51" s="383" t="n"/>
-      <c r="AM51" s="384" t="n"/>
+      <c r="AD51" s="382" t="n"/>
+      <c r="AE51" s="382" t="n"/>
+      <c r="AF51" s="382" t="n"/>
+      <c r="AG51" s="382" t="n"/>
+      <c r="AH51" s="382" t="n"/>
+      <c r="AI51" s="382" t="n"/>
+      <c r="AJ51" s="382" t="n"/>
+      <c r="AK51" s="382" t="n"/>
+      <c r="AL51" s="382" t="n"/>
+      <c r="AM51" s="383" t="n"/>
       <c r="AN51" s="155" t="n"/>
       <c r="AO51" s="340" t="n"/>
       <c r="AP51" s="353" t="n"/>
@@ -8371,7 +8370,7 @@
       <c r="D52" s="146" t="n">
         <v>38</v>
       </c>
-      <c r="E52" s="385" t="inlineStr">
+      <c r="E52" s="384" t="inlineStr">
         <is>
           <t>Recuperación  del Impto. Específico al Petróleo Diesel (Art. 7º Ley 18.502 y 3º D.S. Nº 311/86)</t>
         </is>
@@ -8423,8 +8422,8 @@
       </c>
       <c r="AO52" s="342" t="n"/>
       <c r="AP52" s="375" t="n"/>
-      <c r="AQ52" s="386" t="n"/>
-      <c r="AR52" s="387" t="n"/>
+      <c r="AQ52" s="385" t="n"/>
+      <c r="AR52" s="386" t="n"/>
       <c r="AS52" s="24" t="inlineStr">
         <is>
           <t>+</t>
@@ -8479,9 +8478,9 @@
       <c r="AM53" s="340" t="n"/>
       <c r="AN53" s="344" t="n"/>
       <c r="AO53" s="346" t="n"/>
-      <c r="AP53" s="388" t="n"/>
-      <c r="AQ53" s="389" t="n"/>
-      <c r="AR53" s="390" t="n"/>
+      <c r="AP53" s="387" t="n"/>
+      <c r="AQ53" s="388" t="n"/>
+      <c r="AR53" s="389" t="n"/>
       <c r="AS53" s="347" t="n"/>
     </row>
     <row r="54" ht="27.75" customHeight="1">
@@ -8491,7 +8490,7 @@
       <c r="D54" s="146" t="n">
         <v>39</v>
       </c>
-      <c r="E54" s="385" t="inlineStr">
+      <c r="E54" s="384" t="inlineStr">
         <is>
           <t>Recuperación  del Impto. Específico al Petróleo Diesel soportado por Transportistas de Carga (Art. 2º Ley 19.764)</t>
         </is>
@@ -8543,8 +8542,8 @@
       </c>
       <c r="AO54" s="342" t="n"/>
       <c r="AP54" s="375" t="n"/>
-      <c r="AQ54" s="386" t="n"/>
-      <c r="AR54" s="387" t="n"/>
+      <c r="AQ54" s="385" t="n"/>
+      <c r="AR54" s="386" t="n"/>
       <c r="AS54" s="24" t="inlineStr">
         <is>
           <t>+</t>
@@ -8599,9 +8598,9 @@
       <c r="AM55" s="340" t="n"/>
       <c r="AN55" s="344" t="n"/>
       <c r="AO55" s="346" t="n"/>
-      <c r="AP55" s="388" t="n"/>
-      <c r="AQ55" s="389" t="n"/>
-      <c r="AR55" s="390" t="n"/>
+      <c r="AP55" s="387" t="n"/>
+      <c r="AQ55" s="388" t="n"/>
+      <c r="AR55" s="389" t="n"/>
       <c r="AS55" s="347" t="n"/>
     </row>
     <row r="56" ht="27.75" customHeight="1">
@@ -8611,7 +8610,7 @@
       <c r="D56" s="146" t="n">
         <v>40</v>
       </c>
-      <c r="E56" s="391" t="inlineStr">
+      <c r="E56" s="390" t="inlineStr">
         <is>
           <t>Crédito del Art. 11º Ley 18.211 (correspondiente a Zona Franca de Extensión)</t>
         </is>
@@ -8827,9 +8826,9 @@
       <c r="AN59" s="8" t="n"/>
       <c r="AO59" s="8" t="n"/>
       <c r="AP59" s="8" t="n"/>
-      <c r="AQ59" s="392" t="n"/>
-      <c r="AR59" s="393" t="n"/>
-      <c r="AS59" s="393" t="n"/>
+      <c r="AQ59" s="391" t="n"/>
+      <c r="AR59" s="392" t="n"/>
+      <c r="AS59" s="392" t="n"/>
     </row>
     <row r="60" ht="15.75" customHeight="1">
       <c r="A60" s="8" t="n"/>
@@ -9006,7 +9005,7 @@
         <v>77</v>
       </c>
       <c r="Q63" s="340" t="n"/>
-      <c r="R63" s="394" t="n"/>
+      <c r="R63" s="393" t="n"/>
       <c r="S63" s="349" t="n"/>
       <c r="T63" s="349" t="n"/>
       <c r="U63" s="349" t="n"/>
@@ -9036,7 +9035,7 @@
         <v>89</v>
       </c>
       <c r="AO63" s="340" t="n"/>
-      <c r="AP63" s="395">
+      <c r="AP63" s="394">
         <f>MAX(AP29-AP58,0)</f>
         <v/>
       </c>
@@ -9229,7 +9228,7 @@
         <v>46</v>
       </c>
       <c r="E67" s="355" t="n"/>
-      <c r="F67" s="379" t="inlineStr">
+      <c r="F67" s="378" t="inlineStr">
         <is>
           <t>Retención de Impuesto con tasa del 10% sobre las rentas del Art. 42 Nº2, según Art. 74 Nº2 LIR</t>
         </is>
@@ -9631,7 +9630,7 @@
       <c r="AK73" s="339" t="n"/>
       <c r="AL73" s="339" t="n"/>
       <c r="AM73" s="340" t="n"/>
-      <c r="AN73" s="396" t="inlineStr">
+      <c r="AN73" s="395" t="inlineStr">
         <is>
           <t>PPM Neto Determinado</t>
         </is>
@@ -9664,7 +9663,7 @@
       <c r="I74" s="175" t="n">
         <v>30</v>
       </c>
-      <c r="J74" s="397" t="n"/>
+      <c r="J74" s="396" t="n"/>
       <c r="K74" s="349" t="n"/>
       <c r="L74" s="349" t="n"/>
       <c r="M74" s="349" t="n"/>
@@ -9675,7 +9674,7 @@
       <c r="R74" s="153" t="n">
         <v>563</v>
       </c>
-      <c r="S74" s="398">
+      <c r="S74" s="397">
         <f>'L. VENTAS'!C81</f>
         <v/>
       </c>
@@ -9690,7 +9689,7 @@
         <v>115</v>
       </c>
       <c r="AB74" s="340" t="n"/>
-      <c r="AC74" s="399">
+      <c r="AC74" s="398">
         <f>'L. VENTAS'!A81</f>
         <v/>
       </c>
@@ -9699,7 +9698,7 @@
         <v>68</v>
       </c>
       <c r="AF74" s="340" t="n"/>
-      <c r="AG74" s="400" t="n"/>
+      <c r="AG74" s="399" t="n"/>
       <c r="AH74" s="349" t="n"/>
       <c r="AI74" s="349" t="n"/>
       <c r="AJ74" s="349" t="n"/>
@@ -9710,7 +9709,7 @@
         <v>62</v>
       </c>
       <c r="AO74" s="340" t="n"/>
-      <c r="AP74" s="401">
+      <c r="AP74" s="400">
         <f>'L. VENTAS'!D81</f>
         <v/>
       </c>
@@ -9740,7 +9739,7 @@
       <c r="I75" s="175" t="n">
         <v>565</v>
       </c>
-      <c r="J75" s="397" t="n"/>
+      <c r="J75" s="396" t="n"/>
       <c r="K75" s="349" t="n"/>
       <c r="L75" s="349" t="n"/>
       <c r="M75" s="349" t="n"/>
@@ -9751,7 +9750,7 @@
       <c r="R75" s="175" t="n">
         <v>120</v>
       </c>
-      <c r="S75" s="402" t="n"/>
+      <c r="S75" s="401" t="n"/>
       <c r="T75" s="349" t="n"/>
       <c r="U75" s="349" t="n"/>
       <c r="V75" s="349" t="n"/>
@@ -9763,13 +9762,13 @@
         <v>542</v>
       </c>
       <c r="AB75" s="340" t="n"/>
-      <c r="AC75" s="399" t="n"/>
+      <c r="AC75" s="398" t="n"/>
       <c r="AD75" s="350" t="n"/>
       <c r="AE75" s="175" t="n">
         <v>122</v>
       </c>
       <c r="AF75" s="340" t="n"/>
-      <c r="AG75" s="400" t="n"/>
+      <c r="AG75" s="399" t="n"/>
       <c r="AH75" s="349" t="n"/>
       <c r="AI75" s="349" t="n"/>
       <c r="AJ75" s="349" t="n"/>
@@ -9807,7 +9806,7 @@
       <c r="I76" s="175" t="n">
         <v>700</v>
       </c>
-      <c r="J76" s="397" t="n"/>
+      <c r="J76" s="396" t="n"/>
       <c r="K76" s="349" t="n"/>
       <c r="L76" s="349" t="n"/>
       <c r="M76" s="349" t="n"/>
@@ -9818,7 +9817,7 @@
       <c r="R76" s="175" t="n">
         <v>701</v>
       </c>
-      <c r="S76" s="402" t="n"/>
+      <c r="S76" s="401" t="n"/>
       <c r="T76" s="349" t="n"/>
       <c r="U76" s="349" t="n"/>
       <c r="V76" s="349" t="n"/>
@@ -9830,13 +9829,13 @@
         <v>702</v>
       </c>
       <c r="AB76" s="340" t="n"/>
-      <c r="AC76" s="399" t="n"/>
+      <c r="AC76" s="398" t="n"/>
       <c r="AD76" s="350" t="n"/>
       <c r="AE76" s="175" t="n">
         <v>711</v>
       </c>
       <c r="AF76" s="340" t="n"/>
-      <c r="AG76" s="400" t="n"/>
+      <c r="AG76" s="399" t="n"/>
       <c r="AH76" s="349" t="n"/>
       <c r="AI76" s="349" t="n"/>
       <c r="AJ76" s="349" t="n"/>
@@ -9923,56 +9922,56 @@
         <v>56</v>
       </c>
       <c r="E78" s="355" t="n"/>
-      <c r="F78" s="403" t="inlineStr">
+      <c r="F78" s="402" t="inlineStr">
         <is>
           <t>Crédito Capacitación</t>
         </is>
       </c>
-      <c r="G78" s="404" t="n"/>
-      <c r="H78" s="405" t="n"/>
+      <c r="G78" s="403" t="n"/>
+      <c r="H78" s="404" t="n"/>
       <c r="I78" s="278" t="inlineStr">
         <is>
           <t>Crédito del mes</t>
         </is>
       </c>
-      <c r="J78" s="383" t="n"/>
-      <c r="K78" s="383" t="n"/>
-      <c r="L78" s="383" t="n"/>
-      <c r="M78" s="383" t="n"/>
-      <c r="N78" s="383" t="n"/>
-      <c r="O78" s="383" t="n"/>
-      <c r="P78" s="383" t="n"/>
-      <c r="Q78" s="384" t="n"/>
+      <c r="J78" s="382" t="n"/>
+      <c r="K78" s="382" t="n"/>
+      <c r="L78" s="382" t="n"/>
+      <c r="M78" s="382" t="n"/>
+      <c r="N78" s="382" t="n"/>
+      <c r="O78" s="382" t="n"/>
+      <c r="P78" s="382" t="n"/>
+      <c r="Q78" s="383" t="n"/>
       <c r="R78" s="278" t="inlineStr">
         <is>
           <t>Remanente mes Anterior</t>
         </is>
       </c>
-      <c r="S78" s="383" t="n"/>
-      <c r="T78" s="383" t="n"/>
-      <c r="U78" s="383" t="n"/>
-      <c r="V78" s="383" t="n"/>
-      <c r="W78" s="383" t="n"/>
-      <c r="X78" s="383" t="n"/>
-      <c r="Y78" s="383" t="n"/>
-      <c r="Z78" s="384" t="n"/>
+      <c r="S78" s="382" t="n"/>
+      <c r="T78" s="382" t="n"/>
+      <c r="U78" s="382" t="n"/>
+      <c r="V78" s="382" t="n"/>
+      <c r="W78" s="382" t="n"/>
+      <c r="X78" s="382" t="n"/>
+      <c r="Y78" s="382" t="n"/>
+      <c r="Z78" s="383" t="n"/>
       <c r="AA78" s="278" t="inlineStr">
         <is>
           <t>Remanente Período sgte</t>
         </is>
       </c>
-      <c r="AB78" s="383" t="n"/>
-      <c r="AC78" s="383" t="n"/>
-      <c r="AD78" s="383" t="n"/>
-      <c r="AE78" s="383" t="n"/>
-      <c r="AF78" s="383" t="n"/>
-      <c r="AG78" s="384" t="n"/>
+      <c r="AB78" s="382" t="n"/>
+      <c r="AC78" s="382" t="n"/>
+      <c r="AD78" s="382" t="n"/>
+      <c r="AE78" s="382" t="n"/>
+      <c r="AF78" s="382" t="n"/>
+      <c r="AG78" s="383" t="n"/>
       <c r="AH78" s="278" t="n"/>
-      <c r="AI78" s="383" t="n"/>
-      <c r="AJ78" s="383" t="n"/>
-      <c r="AK78" s="383" t="n"/>
-      <c r="AL78" s="383" t="n"/>
-      <c r="AM78" s="384" t="n"/>
+      <c r="AI78" s="382" t="n"/>
+      <c r="AJ78" s="382" t="n"/>
+      <c r="AK78" s="382" t="n"/>
+      <c r="AL78" s="382" t="n"/>
+      <c r="AM78" s="383" t="n"/>
       <c r="AN78" s="146" t="n"/>
       <c r="AO78" s="340" t="n"/>
       <c r="AP78" s="353" t="n"/>
@@ -9986,13 +9985,13 @@
       <c r="C79" s="352" t="n"/>
       <c r="D79" s="355" t="n"/>
       <c r="E79" s="355" t="n"/>
-      <c r="F79" s="406" t="inlineStr">
+      <c r="F79" s="405" t="inlineStr">
         <is>
           <t>Ley 19.518/97</t>
         </is>
       </c>
-      <c r="G79" s="407" t="n"/>
-      <c r="H79" s="408" t="n"/>
+      <c r="G79" s="406" t="n"/>
+      <c r="H79" s="407" t="n"/>
       <c r="I79" s="175" t="n">
         <v>721</v>
       </c>
@@ -10018,7 +10017,7 @@
       <c r="AA79" s="278" t="n">
         <v>724</v>
       </c>
-      <c r="AB79" s="384" t="n"/>
+      <c r="AB79" s="383" t="n"/>
       <c r="AC79" s="99" t="n"/>
       <c r="AD79" s="99" t="n"/>
       <c r="AE79" s="99" t="n"/>
@@ -10029,11 +10028,11 @@
           <t>Crédito a imutar</t>
         </is>
       </c>
-      <c r="AI79" s="404" t="n"/>
-      <c r="AJ79" s="404" t="n"/>
-      <c r="AK79" s="404" t="n"/>
-      <c r="AL79" s="404" t="n"/>
-      <c r="AM79" s="405" t="n"/>
+      <c r="AI79" s="403" t="n"/>
+      <c r="AJ79" s="403" t="n"/>
+      <c r="AK79" s="403" t="n"/>
+      <c r="AL79" s="403" t="n"/>
+      <c r="AM79" s="404" t="n"/>
       <c r="AN79" s="155" t="n">
         <v>723</v>
       </c>
@@ -10262,7 +10261,7 @@
         <v>595</v>
       </c>
       <c r="AO83" s="340" t="n"/>
-      <c r="AP83" s="401">
+      <c r="AP83" s="400">
         <f>AP63+AP74</f>
         <v/>
       </c>
@@ -10323,7 +10322,7 @@
     </row>
     <row r="85" ht="15.75" customHeight="1">
       <c r="A85" s="8" t="n"/>
-      <c r="B85" s="391" t="inlineStr">
+      <c r="B85" s="390" t="inlineStr">
         <is>
           <t xml:space="preserve">Si no declara Tributación Simplificada, Impuesto Adicional (Art. 37 o Art. 42), Cotización Adicional, Crédito Especial Empresas Constructoras, Recuperación de Peaje Transportistas de Pasajeros o Cambio de Sujeto; traslade el valor a línea 47 (código 595) </t>
         </is>
@@ -10475,7 +10474,7 @@
           <t>05</t>
         </is>
       </c>
-      <c r="AJ87" s="396" t="inlineStr">
+      <c r="AJ87" s="395" t="inlineStr">
         <is>
           <t>Nombres</t>
         </is>
@@ -10492,7 +10491,7 @@
     </row>
     <row r="88" ht="23.25" customHeight="1">
       <c r="A88" s="8" t="n"/>
-      <c r="B88" s="409" t="inlineStr">
+      <c r="B88" s="408" t="inlineStr">
         <is>
           <t>Silvestres del Ñuble SpA (ficticia)</t>
         </is>
@@ -10559,8 +10558,8 @@
       <c r="K89" s="146" t="n">
         <v>583</v>
       </c>
-      <c r="L89" s="410" t="n"/>
-      <c r="M89" s="411" t="n"/>
+      <c r="L89" s="409" t="n"/>
+      <c r="M89" s="410" t="n"/>
       <c r="N89" s="8" t="n"/>
       <c r="O89" s="8" t="n"/>
       <c r="P89" s="8" t="n"/>
@@ -10610,8 +10609,8 @@
       <c r="I90" s="345" t="n"/>
       <c r="J90" s="346" t="n"/>
       <c r="K90" s="347" t="n"/>
-      <c r="L90" s="412" t="n"/>
-      <c r="M90" s="413" t="n"/>
+      <c r="L90" s="411" t="n"/>
+      <c r="M90" s="412" t="n"/>
       <c r="N90" s="8" t="inlineStr">
         <is>
           <t>(Si marca con X el casillero, registre los cambios al reverso)</t>
@@ -10698,7 +10697,7 @@
     </row>
     <row r="92" ht="18.75" customHeight="1">
       <c r="A92" s="8" t="n"/>
-      <c r="B92" s="391" t="inlineStr">
+      <c r="B92" s="390" t="inlineStr">
         <is>
           <t>Declaro bajo juramento que los datos contenidos en esta declaración son la expresión fiel de la verdad, por lo que asumo la responsabilidad correspondiente.</t>
         </is>
@@ -10750,7 +10749,7 @@
         <v>91</v>
       </c>
       <c r="AO92" s="340" t="n"/>
-      <c r="AP92" s="401">
+      <c r="AP92" s="400">
         <f>AP83+AP100</f>
         <v/>
       </c>
@@ -10765,17 +10764,17 @@
     <row r="93" ht="18.75" customHeight="1">
       <c r="A93" s="8" t="n"/>
       <c r="B93" s="351" t="n"/>
-      <c r="C93" s="393" t="n"/>
-      <c r="D93" s="393" t="n"/>
-      <c r="E93" s="393" t="n"/>
-      <c r="F93" s="393" t="n"/>
-      <c r="G93" s="393" t="n"/>
-      <c r="H93" s="393" t="n"/>
-      <c r="I93" s="393" t="n"/>
-      <c r="J93" s="393" t="n"/>
-      <c r="K93" s="393" t="n"/>
-      <c r="L93" s="393" t="n"/>
-      <c r="M93" s="393" t="n"/>
+      <c r="C93" s="392" t="n"/>
+      <c r="D93" s="392" t="n"/>
+      <c r="E93" s="392" t="n"/>
+      <c r="F93" s="392" t="n"/>
+      <c r="G93" s="392" t="n"/>
+      <c r="H93" s="392" t="n"/>
+      <c r="I93" s="392" t="n"/>
+      <c r="J93" s="392" t="n"/>
+      <c r="K93" s="392" t="n"/>
+      <c r="L93" s="392" t="n"/>
+      <c r="M93" s="392" t="n"/>
       <c r="N93" s="352" t="n"/>
       <c r="O93" s="8" t="n"/>
       <c r="P93" s="8" t="n"/>
@@ -10949,7 +10948,7 @@
     <row r="97">
       <c r="B97" t="inlineStr">
         <is>
-          <t>[39] Retenciones de IVA a terceros con retención total (línea 118 en las instrucciones de nov-2024; el N° de línea cambia según el año) ⚠️</t>
+          <t>[39] Retenciones de IVA a terceros con retención total (línea 118 en las instrucciones SII del 12-11-2024)</t>
         </is>
       </c>
       <c r="AP97" s="47">
@@ -10988,7 +10987,7 @@
     <row r="102">
       <c r="B102" t="inlineStr">
         <is>
-          <t>Amarillo: línea 5 (retención total, vendedor retenido), líneas 6 y 14 (retención parcial, vendedor retenido) y línea 22 (compras sin derecho a crédito fiscal: la factura de compra del agente retenedor, códigos 564 y 521).</t>
+          <t>Amarillo: línea 5 (retención total, vendedor retenido), líneas 6 y 14 (retención parcial, vendedor retenido) y línea 25 (facturas de compra emitidas por el agente retenedor, con derecho a crédito: códigos 519 y 520). En las instrucciones SII del 12-11-2024 estas líneas son la 5, 6, 16 y 28.</t>
         </is>
       </c>
     </row>
@@ -11408,7 +11407,7 @@
       <c r="E2" s="6" t="n"/>
     </row>
     <row r="3" ht="18.75" customHeight="1">
-      <c r="B3" s="414" t="n"/>
+      <c r="B3" s="413" t="n"/>
       <c r="C3" s="315" t="n">
         <v>2024</v>
       </c>
@@ -11641,7 +11640,7 @@
           <t>Empresa (ficticia)</t>
         </is>
       </c>
-      <c r="B1" s="415" t="inlineStr">
+      <c r="B1" s="414" t="inlineStr">
         <is>
           <t>Silvestres del Ñuble SpA (ficticia)</t>
         </is>
@@ -11653,7 +11652,7 @@
           <t>RUT (ficticio)</t>
         </is>
       </c>
-      <c r="B2" s="415" t="inlineStr">
+      <c r="B2" s="414" t="inlineStr">
         <is>
           <t>76.123.456-0</t>
         </is>
@@ -11665,7 +11664,7 @@
           <t>Período</t>
         </is>
       </c>
-      <c r="B3" s="415" t="inlineStr">
+      <c r="B3" s="414" t="inlineStr">
         <is>
           <t>Octubre 2026</t>
         </is>
@@ -11677,7 +11676,7 @@
           <t>Tasa de IVA</t>
         </is>
       </c>
-      <c r="B4" s="416" t="n">
+      <c r="B4" s="415" t="n">
         <v>0.19</v>
       </c>
     </row>
@@ -11687,7 +11686,7 @@
           <t>Retención del IVA (1 = total; Res. Ex. SII 4095/2000)</t>
         </is>
       </c>
-      <c r="B5" s="416" t="n">
+      <c r="B5" s="415" t="n">
         <v>1</v>
       </c>
     </row>
@@ -11697,7 +11696,7 @@
           <t>Margen de ganancia sobre el costo</t>
         </is>
       </c>
-      <c r="B6" s="416" t="n">
+      <c r="B6" s="415" t="n">
         <v>0.4</v>
       </c>
     </row>
@@ -11707,7 +11706,7 @@
           <t>Integrantes</t>
         </is>
       </c>
-      <c r="B7" s="415" t="inlineStr">
+      <c r="B7" s="414" t="inlineStr">
         <is>
           <t>Matius Loyola, Diego Quintana, Joaquín Verdejo</t>
         </is>
@@ -11756,93 +11755,93 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="417" t="inlineStr">
+      <c r="A4" s="416" t="inlineStr">
         <is>
           <t>Folio</t>
         </is>
       </c>
-      <c r="B4" s="417" t="inlineStr">
+      <c r="B4" s="416" t="inlineStr">
         <is>
           <t>Fecha</t>
         </is>
       </c>
-      <c r="C4" s="417" t="inlineStr">
+      <c r="C4" s="416" t="inlineStr">
         <is>
           <t>Proveedor</t>
         </is>
       </c>
-      <c r="D4" s="417" t="inlineStr">
+      <c r="D4" s="416" t="inlineStr">
         <is>
           <t>RUT</t>
         </is>
       </c>
-      <c r="E4" s="417" t="inlineStr">
+      <c r="E4" s="416" t="inlineStr">
         <is>
           <t>Producto</t>
         </is>
       </c>
-      <c r="F4" s="417" t="inlineStr">
+      <c r="F4" s="416" t="inlineStr">
         <is>
           <t>Kilos</t>
         </is>
       </c>
-      <c r="G4" s="417" t="inlineStr">
+      <c r="G4" s="416" t="inlineStr">
         <is>
           <t>Precio por kilo</t>
         </is>
       </c>
-      <c r="H4" s="417" t="inlineStr">
+      <c r="H4" s="416" t="inlineStr">
         <is>
           <t>Neto</t>
         </is>
       </c>
-      <c r="I4" s="417" t="inlineStr">
+      <c r="I4" s="416" t="inlineStr">
         <is>
           <t>IVA 19 %</t>
         </is>
       </c>
-      <c r="J4" s="417" t="inlineStr">
+      <c r="J4" s="416" t="inlineStr">
         <is>
           <t>IVA retenido</t>
         </is>
       </c>
-      <c r="K4" s="417" t="inlineStr">
+      <c r="K4" s="416" t="inlineStr">
         <is>
           <t>IVA que cobra el proveedor</t>
         </is>
       </c>
-      <c r="L4" s="417" t="inlineStr">
+      <c r="L4" s="416" t="inlineStr">
         <is>
           <t>Total a pagar al proveedor</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="415" t="n">
+      <c r="A5" s="414" t="n">
         <v>201</v>
       </c>
-      <c r="B5" s="418" t="n">
+      <c r="B5" s="417" t="n">
         <v>46297</v>
       </c>
-      <c r="C5" s="415" t="inlineStr">
+      <c r="C5" s="414" t="inlineStr">
         <is>
           <t>Juan Pérez (recolector)</t>
         </is>
       </c>
-      <c r="D5" s="415" t="inlineStr">
+      <c r="D5" s="414" t="inlineStr">
         <is>
           <t>11.111.111-1</t>
         </is>
       </c>
-      <c r="E5" s="415" t="inlineStr">
+      <c r="E5" s="414" t="inlineStr">
         <is>
           <t>Rosa mosqueta</t>
         </is>
       </c>
-      <c r="F5" s="419" t="n">
+      <c r="F5" s="418" t="n">
         <v>1200</v>
       </c>
-      <c r="G5" s="419" t="n">
+      <c r="G5" s="418" t="n">
         <v>1500</v>
       </c>
       <c r="H5" s="47">
@@ -11867,31 +11866,31 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="415" t="n">
+      <c r="A6" s="414" t="n">
         <v>202</v>
       </c>
-      <c r="B6" s="418" t="n">
+      <c r="B6" s="417" t="n">
         <v>46301</v>
       </c>
-      <c r="C6" s="415" t="inlineStr">
+      <c r="C6" s="414" t="inlineStr">
         <is>
           <t>María Soto (recolectora)</t>
         </is>
       </c>
-      <c r="D6" s="415" t="inlineStr">
+      <c r="D6" s="414" t="inlineStr">
         <is>
           <t>12.222.222-5</t>
         </is>
       </c>
-      <c r="E6" s="415" t="inlineStr">
+      <c r="E6" s="414" t="inlineStr">
         <is>
           <t>Hongos</t>
         </is>
       </c>
-      <c r="F6" s="419" t="n">
+      <c r="F6" s="418" t="n">
         <v>300</v>
       </c>
-      <c r="G6" s="419" t="n">
+      <c r="G6" s="418" t="n">
         <v>4000</v>
       </c>
       <c r="H6" s="47">
@@ -11916,31 +11915,31 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="415" t="n">
+      <c r="A7" s="414" t="n">
         <v>203</v>
       </c>
-      <c r="B7" s="418" t="n">
+      <c r="B7" s="417" t="n">
         <v>46307</v>
       </c>
-      <c r="C7" s="415" t="inlineStr">
+      <c r="C7" s="414" t="inlineStr">
         <is>
           <t>Pedro Núñez (recolector)</t>
         </is>
       </c>
-      <c r="D7" s="415" t="inlineStr">
+      <c r="D7" s="414" t="inlineStr">
         <is>
           <t>13.333.333-9</t>
         </is>
       </c>
-      <c r="E7" s="415" t="inlineStr">
+      <c r="E7" s="414" t="inlineStr">
         <is>
           <t>Mora</t>
         </is>
       </c>
-      <c r="F7" s="419" t="n">
+      <c r="F7" s="418" t="n">
         <v>500</v>
       </c>
-      <c r="G7" s="419" t="n">
+      <c r="G7" s="418" t="n">
         <v>1600</v>
       </c>
       <c r="H7" s="47">
@@ -11965,31 +11964,31 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="415" t="n">
+      <c r="A8" s="414" t="n">
         <v>204</v>
       </c>
-      <c r="B8" s="418" t="n">
+      <c r="B8" s="417" t="n">
         <v>46314</v>
       </c>
-      <c r="C8" s="415" t="inlineStr">
+      <c r="C8" s="414" t="inlineStr">
         <is>
           <t>Rosa Muñoz (recolectora)</t>
         </is>
       </c>
-      <c r="D8" s="415" t="inlineStr">
+      <c r="D8" s="414" t="inlineStr">
         <is>
           <t>14.444.444-2</t>
         </is>
       </c>
-      <c r="E8" s="415" t="inlineStr">
+      <c r="E8" s="414" t="inlineStr">
         <is>
           <t>Hojas de boldo</t>
         </is>
       </c>
-      <c r="F8" s="419" t="n">
+      <c r="F8" s="418" t="n">
         <v>400</v>
       </c>
-      <c r="G8" s="419" t="n">
+      <c r="G8" s="418" t="n">
         <v>1250</v>
       </c>
       <c r="H8" s="47">
@@ -12014,31 +12013,31 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="415" t="n">
+      <c r="A9" s="414" t="n">
         <v>205</v>
       </c>
-      <c r="B9" s="418" t="n">
+      <c r="B9" s="417" t="n">
         <v>46321</v>
       </c>
-      <c r="C9" s="415" t="inlineStr">
+      <c r="C9" s="414" t="inlineStr">
         <is>
           <t>Luis Araya (recolector)</t>
         </is>
       </c>
-      <c r="D9" s="415" t="inlineStr">
+      <c r="D9" s="414" t="inlineStr">
         <is>
           <t>15.555.555-6</t>
         </is>
       </c>
-      <c r="E9" s="415" t="inlineStr">
+      <c r="E9" s="414" t="inlineStr">
         <is>
           <t>Frutos de espino</t>
         </is>
       </c>
-      <c r="F9" s="419" t="n">
+      <c r="F9" s="418" t="n">
         <v>900</v>
       </c>
-      <c r="G9" s="419" t="n">
+      <c r="G9" s="418" t="n">
         <v>1500</v>
       </c>
       <c r="H9" s="47">
@@ -12100,7 +12099,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G40"/>
+  <dimension ref="A1:G46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -12113,32 +12112,32 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="420" t="inlineStr">
+      <c r="A1" s="419" t="inlineStr">
         <is>
           <t>Asiento</t>
         </is>
       </c>
-      <c r="B1" s="420" t="inlineStr">
+      <c r="B1" s="419" t="inlineStr">
         <is>
           <t>Fecha</t>
         </is>
       </c>
-      <c r="C1" s="420" t="inlineStr">
+      <c r="C1" s="419" t="inlineStr">
         <is>
           <t>Cuenta</t>
         </is>
       </c>
-      <c r="D1" s="420" t="inlineStr">
+      <c r="D1" s="419" t="inlineStr">
         <is>
           <t>Glosa</t>
         </is>
       </c>
-      <c r="E1" s="420" t="inlineStr">
+      <c r="E1" s="419" t="inlineStr">
         <is>
           <t>Debe</t>
         </is>
       </c>
-      <c r="F1" s="420" t="inlineStr">
+      <c r="F1" s="419" t="inlineStr">
         <is>
           <t>Haber</t>
         </is>
@@ -12148,7 +12147,7 @@
       <c r="A2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="421" t="n">
+      <c r="B2" s="420" t="n">
         <v>46297</v>
       </c>
       <c r="C2" t="inlineStr">
@@ -12162,7 +12161,7 @@
         </is>
       </c>
       <c r="E2" s="47">
-        <f>'L. COMPRAS'!H7+'L. COMPRAS'!I7</f>
+        <f>'L. COMPRAS'!H7</f>
         <v/>
       </c>
     </row>
@@ -12170,12 +12169,12 @@
       <c r="A3" t="n">
         <v>1</v>
       </c>
-      <c r="B3" s="421" t="n">
+      <c r="B3" s="420" t="n">
         <v>46297</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2.1.01 Proveedores</t>
+          <t>1.1.04 IVA crédito fiscal</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -12183,8 +12182,8 @@
           <t>Factura de compra N°201: Rosa mosqueta (IVA retenido)</t>
         </is>
       </c>
-      <c r="F3" s="47">
-        <f>'L. COMPRAS'!J7-'L. COMPRAS'!K7</f>
+      <c r="E3" s="47">
+        <f>'L. COMPRAS'!I7</f>
         <v/>
       </c>
     </row>
@@ -12192,12 +12191,12 @@
       <c r="A4" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="421" t="n">
+      <c r="B4" s="420" t="n">
         <v>46297</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2.1.09 IVA retenido por pagar</t>
+          <t>2.1.01 Proveedores</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -12206,29 +12205,29 @@
         </is>
       </c>
       <c r="F4" s="47">
-        <f>'L. COMPRAS'!K7</f>
+        <f>'L. COMPRAS'!J7-'L. COMPRAS'!K7</f>
         <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>2</v>
-      </c>
-      <c r="B5" s="421" t="n">
-        <v>46301</v>
+        <v>1</v>
+      </c>
+      <c r="B5" s="420" t="n">
+        <v>46297</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>1.1.13 Inventario mercaderías</t>
+          <t>2.1.09 IVA retenido por pagar</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Factura de compra N°202: Hongos (IVA retenido)</t>
-        </is>
-      </c>
-      <c r="E5" s="47">
-        <f>'L. COMPRAS'!H8+'L. COMPRAS'!I8</f>
+          <t>Factura de compra N°201: Rosa mosqueta (IVA retenido)</t>
+        </is>
+      </c>
+      <c r="F5" s="47">
+        <f>'L. COMPRAS'!K7</f>
         <v/>
       </c>
     </row>
@@ -12236,12 +12235,12 @@
       <c r="A6" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="421" t="n">
+      <c r="B6" s="420" t="n">
         <v>46301</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2.1.01 Proveedores</t>
+          <t>1.1.13 Inventario mercaderías</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -12249,8 +12248,8 @@
           <t>Factura de compra N°202: Hongos (IVA retenido)</t>
         </is>
       </c>
-      <c r="F6" s="47">
-        <f>'L. COMPRAS'!J8-'L. COMPRAS'!K8</f>
+      <c r="E6" s="47">
+        <f>'L. COMPRAS'!H8</f>
         <v/>
       </c>
     </row>
@@ -12258,12 +12257,12 @@
       <c r="A7" t="n">
         <v>2</v>
       </c>
-      <c r="B7" s="421" t="n">
+      <c r="B7" s="420" t="n">
         <v>46301</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2.1.09 IVA retenido por pagar</t>
+          <t>1.1.04 IVA crédito fiscal</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -12271,52 +12270,52 @@
           <t>Factura de compra N°202: Hongos (IVA retenido)</t>
         </is>
       </c>
-      <c r="F7" s="47">
-        <f>'L. COMPRAS'!K8</f>
+      <c r="E7" s="47">
+        <f>'L. COMPRAS'!I8</f>
         <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>3</v>
-      </c>
-      <c r="B8" s="421" t="n">
-        <v>46307</v>
+        <v>2</v>
+      </c>
+      <c r="B8" s="420" t="n">
+        <v>46301</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>1.1.13 Inventario mercaderías</t>
+          <t>2.1.01 Proveedores</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Factura de compra N°203: Mora (IVA retenido)</t>
-        </is>
-      </c>
-      <c r="E8" s="47">
-        <f>'L. COMPRAS'!H9+'L. COMPRAS'!I9</f>
+          <t>Factura de compra N°202: Hongos (IVA retenido)</t>
+        </is>
+      </c>
+      <c r="F8" s="47">
+        <f>'L. COMPRAS'!J8-'L. COMPRAS'!K8</f>
         <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>3</v>
-      </c>
-      <c r="B9" s="421" t="n">
-        <v>46307</v>
+        <v>2</v>
+      </c>
+      <c r="B9" s="420" t="n">
+        <v>46301</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2.1.01 Proveedores</t>
+          <t>2.1.09 IVA retenido por pagar</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Factura de compra N°203: Mora (IVA retenido)</t>
+          <t>Factura de compra N°202: Hongos (IVA retenido)</t>
         </is>
       </c>
       <c r="F9" s="47">
-        <f>'L. COMPRAS'!J9-'L. COMPRAS'!K9</f>
+        <f>'L. COMPRAS'!K8</f>
         <v/>
       </c>
     </row>
@@ -12324,12 +12323,12 @@
       <c r="A10" t="n">
         <v>3</v>
       </c>
-      <c r="B10" s="421" t="n">
+      <c r="B10" s="420" t="n">
         <v>46307</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2.1.09 IVA retenido por pagar</t>
+          <t>1.1.13 Inventario mercaderías</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -12337,39 +12336,39 @@
           <t>Factura de compra N°203: Mora (IVA retenido)</t>
         </is>
       </c>
-      <c r="F10" s="47">
-        <f>'L. COMPRAS'!K9</f>
+      <c r="E10" s="47">
+        <f>'L. COMPRAS'!H9</f>
         <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>4</v>
-      </c>
-      <c r="B11" s="421" t="n">
-        <v>46314</v>
+        <v>3</v>
+      </c>
+      <c r="B11" s="420" t="n">
+        <v>46307</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1.1.13 Inventario mercaderías</t>
+          <t>1.1.04 IVA crédito fiscal</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Factura de compra N°204: Hojas de boldo (IVA retenido)</t>
+          <t>Factura de compra N°203: Mora (IVA retenido)</t>
         </is>
       </c>
       <c r="E11" s="47">
-        <f>'L. COMPRAS'!H10+'L. COMPRAS'!I10</f>
+        <f>'L. COMPRAS'!I9</f>
         <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>4</v>
-      </c>
-      <c r="B12" s="421" t="n">
-        <v>46314</v>
+        <v>3</v>
+      </c>
+      <c r="B12" s="420" t="n">
+        <v>46307</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -12378,20 +12377,20 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Factura de compra N°204: Hojas de boldo (IVA retenido)</t>
+          <t>Factura de compra N°203: Mora (IVA retenido)</t>
         </is>
       </c>
       <c r="F12" s="47">
-        <f>'L. COMPRAS'!J10-'L. COMPRAS'!K10</f>
+        <f>'L. COMPRAS'!J9-'L. COMPRAS'!K9</f>
         <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>4</v>
-      </c>
-      <c r="B13" s="421" t="n">
-        <v>46314</v>
+        <v>3</v>
+      </c>
+      <c r="B13" s="420" t="n">
+        <v>46307</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -12400,20 +12399,20 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Factura de compra N°204: Hojas de boldo (IVA retenido)</t>
+          <t>Factura de compra N°203: Mora (IVA retenido)</t>
         </is>
       </c>
       <c r="F13" s="47">
-        <f>'L. COMPRAS'!K10</f>
+        <f>'L. COMPRAS'!K9</f>
         <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>5</v>
-      </c>
-      <c r="B14" s="421" t="n">
-        <v>46321</v>
+        <v>4</v>
+      </c>
+      <c r="B14" s="420" t="n">
+        <v>46314</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -12422,482 +12421,482 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Factura de compra N°205: Frutos de espino (IVA retenido)</t>
+          <t>Factura de compra N°204: Hojas de boldo (IVA retenido)</t>
         </is>
       </c>
       <c r="E14" s="47">
-        <f>'L. COMPRAS'!H11+'L. COMPRAS'!I11</f>
+        <f>'L. COMPRAS'!H10</f>
         <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>5</v>
-      </c>
-      <c r="B15" s="421" t="n">
-        <v>46321</v>
+        <v>4</v>
+      </c>
+      <c r="B15" s="420" t="n">
+        <v>46314</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2.1.01 Proveedores</t>
+          <t>1.1.04 IVA crédito fiscal</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Factura de compra N°205: Frutos de espino (IVA retenido)</t>
-        </is>
-      </c>
-      <c r="F15" s="47">
-        <f>'L. COMPRAS'!J11-'L. COMPRAS'!K11</f>
+          <t>Factura de compra N°204: Hojas de boldo (IVA retenido)</t>
+        </is>
+      </c>
+      <c r="E15" s="47">
+        <f>'L. COMPRAS'!I10</f>
         <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>5</v>
-      </c>
-      <c r="B16" s="421" t="n">
-        <v>46321</v>
+        <v>4</v>
+      </c>
+      <c r="B16" s="420" t="n">
+        <v>46314</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2.1.09 IVA retenido por pagar</t>
+          <t>2.1.01 Proveedores</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Factura de compra N°205: Frutos de espino (IVA retenido)</t>
+          <t>Factura de compra N°204: Hojas de boldo (IVA retenido)</t>
         </is>
       </c>
       <c r="F16" s="47">
-        <f>'L. COMPRAS'!K11</f>
+        <f>'L. COMPRAS'!J10-'L. COMPRAS'!K10</f>
         <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>6</v>
-      </c>
-      <c r="B17" s="421" t="n">
-        <v>46300</v>
+        <v>4</v>
+      </c>
+      <c r="B17" s="420" t="n">
+        <v>46314</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>1.1.03 Clientes</t>
+          <t>2.1.09 IVA retenido por pagar</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Factura de venta N°101 a Exportadora Andes SpA</t>
-        </is>
-      </c>
-      <c r="E17" s="47">
-        <f>'L. VENTAS'!J6</f>
+          <t>Factura de compra N°204: Hojas de boldo (IVA retenido)</t>
+        </is>
+      </c>
+      <c r="F17" s="47">
+        <f>'L. COMPRAS'!K10</f>
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>6</v>
-      </c>
-      <c r="B18" s="421" t="n">
-        <v>46300</v>
+        <v>5</v>
+      </c>
+      <c r="B18" s="420" t="n">
+        <v>46321</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>4.1.01 Ventas</t>
+          <t>1.1.13 Inventario mercaderías</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Factura de venta N°101 a Exportadora Andes SpA</t>
-        </is>
-      </c>
-      <c r="F18" s="47">
-        <f>'L. VENTAS'!H6</f>
+          <t>Factura de compra N°205: Frutos de espino (IVA retenido)</t>
+        </is>
+      </c>
+      <c r="E18" s="47">
+        <f>'L. COMPRAS'!H11</f>
         <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>6</v>
-      </c>
-      <c r="B19" s="421" t="n">
-        <v>46300</v>
+        <v>5</v>
+      </c>
+      <c r="B19" s="420" t="n">
+        <v>46321</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2.1.02 IVA débito fiscal</t>
+          <t>1.1.04 IVA crédito fiscal</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Factura de venta N°101 a Exportadora Andes SpA</t>
-        </is>
-      </c>
-      <c r="F19" s="47">
-        <f>'L. VENTAS'!I6</f>
+          <t>Factura de compra N°205: Frutos de espino (IVA retenido)</t>
+        </is>
+      </c>
+      <c r="E19" s="47">
+        <f>'L. COMPRAS'!I11</f>
         <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>7</v>
-      </c>
-      <c r="B20" s="421" t="n">
-        <v>46304</v>
+        <v>5</v>
+      </c>
+      <c r="B20" s="420" t="n">
+        <v>46321</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>1.1.03 Clientes</t>
+          <t>2.1.01 Proveedores</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Factura de venta N°102 a Agroindustrial Sur Ltda.</t>
-        </is>
-      </c>
-      <c r="E20" s="47">
-        <f>'L. VENTAS'!J7</f>
+          <t>Factura de compra N°205: Frutos de espino (IVA retenido)</t>
+        </is>
+      </c>
+      <c r="F20" s="47">
+        <f>'L. COMPRAS'!J11-'L. COMPRAS'!K11</f>
         <v/>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>7</v>
-      </c>
-      <c r="B21" s="421" t="n">
-        <v>46304</v>
+        <v>5</v>
+      </c>
+      <c r="B21" s="420" t="n">
+        <v>46321</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>4.1.01 Ventas</t>
+          <t>2.1.09 IVA retenido por pagar</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Factura de venta N°102 a Agroindustrial Sur Ltda.</t>
+          <t>Factura de compra N°205: Frutos de espino (IVA retenido)</t>
         </is>
       </c>
       <c r="F21" s="47">
-        <f>'L. VENTAS'!H7</f>
+        <f>'L. COMPRAS'!K11</f>
         <v/>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>7</v>
-      </c>
-      <c r="B22" s="421" t="n">
-        <v>46304</v>
+        <v>6</v>
+      </c>
+      <c r="B22" s="420" t="n">
+        <v>46300</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2.1.02 IVA débito fiscal</t>
+          <t>1.1.03 Clientes</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Factura de venta N°102 a Agroindustrial Sur Ltda.</t>
-        </is>
-      </c>
-      <c r="F22" s="47">
-        <f>'L. VENTAS'!I7</f>
+          <t>Factura de venta N°101 a Exportadora Andes SpA</t>
+        </is>
+      </c>
+      <c r="E22" s="47">
+        <f>'L. VENTAS'!J6</f>
         <v/>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>8</v>
-      </c>
-      <c r="B23" s="421" t="n">
-        <v>46309</v>
+        <v>6</v>
+      </c>
+      <c r="B23" s="420" t="n">
+        <v>46300</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>1.1.03 Clientes</t>
+          <t>4.1.01 Ventas</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Factura de venta N°103 a Hierbas del Valle S.A.</t>
-        </is>
-      </c>
-      <c r="E23" s="47">
-        <f>'L. VENTAS'!J8</f>
+          <t>Factura de venta N°101 a Exportadora Andes SpA</t>
+        </is>
+      </c>
+      <c r="F23" s="47">
+        <f>'L. VENTAS'!H6</f>
         <v/>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>8</v>
-      </c>
-      <c r="B24" s="421" t="n">
-        <v>46309</v>
+        <v>6</v>
+      </c>
+      <c r="B24" s="420" t="n">
+        <v>46300</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>4.1.01 Ventas</t>
+          <t>2.1.02 IVA débito fiscal</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Factura de venta N°103 a Hierbas del Valle S.A.</t>
+          <t>Factura de venta N°101 a Exportadora Andes SpA</t>
         </is>
       </c>
       <c r="F24" s="47">
-        <f>'L. VENTAS'!H8</f>
+        <f>'L. VENTAS'!I6</f>
         <v/>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>8</v>
-      </c>
-      <c r="B25" s="421" t="n">
-        <v>46309</v>
+        <v>7</v>
+      </c>
+      <c r="B25" s="420" t="n">
+        <v>46304</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2.1.02 IVA débito fiscal</t>
+          <t>1.1.03 Clientes</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Factura de venta N°103 a Hierbas del Valle S.A.</t>
-        </is>
-      </c>
-      <c r="F25" s="47">
-        <f>'L. VENTAS'!I8</f>
+          <t>Factura de venta N°102 a Agroindustrial Sur Ltda.</t>
+        </is>
+      </c>
+      <c r="E25" s="47">
+        <f>'L. VENTAS'!J7</f>
         <v/>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>9</v>
-      </c>
-      <c r="B26" s="421" t="n">
-        <v>46316</v>
+        <v>7</v>
+      </c>
+      <c r="B26" s="420" t="n">
+        <v>46304</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>1.1.03 Clientes</t>
+          <t>4.1.01 Ventas</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Factura de venta N°104 a Comercial Maule SpA</t>
-        </is>
-      </c>
-      <c r="E26" s="47">
-        <f>'L. VENTAS'!J9</f>
+          <t>Factura de venta N°102 a Agroindustrial Sur Ltda.</t>
+        </is>
+      </c>
+      <c r="F26" s="47">
+        <f>'L. VENTAS'!H7</f>
         <v/>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>9</v>
-      </c>
-      <c r="B27" s="421" t="n">
-        <v>46316</v>
+        <v>7</v>
+      </c>
+      <c r="B27" s="420" t="n">
+        <v>46304</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>4.1.01 Ventas</t>
+          <t>2.1.02 IVA débito fiscal</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Factura de venta N°104 a Comercial Maule SpA</t>
+          <t>Factura de venta N°102 a Agroindustrial Sur Ltda.</t>
         </is>
       </c>
       <c r="F27" s="47">
-        <f>'L. VENTAS'!H9</f>
+        <f>'L. VENTAS'!I7</f>
         <v/>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>9</v>
-      </c>
-      <c r="B28" s="421" t="n">
-        <v>46316</v>
+        <v>8</v>
+      </c>
+      <c r="B28" s="420" t="n">
+        <v>46309</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2.1.02 IVA débito fiscal</t>
+          <t>1.1.03 Clientes</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Factura de venta N°104 a Comercial Maule SpA</t>
-        </is>
-      </c>
-      <c r="F28" s="47">
-        <f>'L. VENTAS'!I9</f>
+          <t>Factura de venta N°103 a Hierbas del Valle S.A.</t>
+        </is>
+      </c>
+      <c r="E28" s="47">
+        <f>'L. VENTAS'!J8</f>
         <v/>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>10</v>
-      </c>
-      <c r="B29" s="421" t="n">
-        <v>46323</v>
+        <v>8</v>
+      </c>
+      <c r="B29" s="420" t="n">
+        <v>46309</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>1.1.03 Clientes</t>
+          <t>4.1.01 Ventas</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Factura de venta N°105 a Distribuidora Bío Bío Ltda.</t>
-        </is>
-      </c>
-      <c r="E29" s="47">
-        <f>'L. VENTAS'!J10</f>
+          <t>Factura de venta N°103 a Hierbas del Valle S.A.</t>
+        </is>
+      </c>
+      <c r="F29" s="47">
+        <f>'L. VENTAS'!H8</f>
         <v/>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>10</v>
-      </c>
-      <c r="B30" s="421" t="n">
-        <v>46323</v>
+        <v>8</v>
+      </c>
+      <c r="B30" s="420" t="n">
+        <v>46309</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>4.1.01 Ventas</t>
+          <t>2.1.02 IVA débito fiscal</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Factura de venta N°105 a Distribuidora Bío Bío Ltda.</t>
+          <t>Factura de venta N°103 a Hierbas del Valle S.A.</t>
         </is>
       </c>
       <c r="F30" s="47">
-        <f>'L. VENTAS'!H10</f>
+        <f>'L. VENTAS'!I8</f>
         <v/>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>10</v>
-      </c>
-      <c r="B31" s="421" t="n">
-        <v>46323</v>
+        <v>9</v>
+      </c>
+      <c r="B31" s="420" t="n">
+        <v>46316</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2.1.02 IVA débito fiscal</t>
+          <t>1.1.03 Clientes</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Factura de venta N°105 a Distribuidora Bío Bío Ltda.</t>
-        </is>
-      </c>
-      <c r="F31" s="47">
-        <f>'L. VENTAS'!I10</f>
+          <t>Factura de venta N°104 a Comercial Maule SpA</t>
+        </is>
+      </c>
+      <c r="E31" s="47">
+        <f>'L. VENTAS'!J9</f>
         <v/>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>11</v>
-      </c>
-      <c r="B32" s="421" t="n">
-        <v>46326</v>
+        <v>9</v>
+      </c>
+      <c r="B32" s="420" t="n">
+        <v>46316</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>5.1.01 Costo de ventas</t>
+          <t>4.1.01 Ventas</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Costo de las ventas del mes</t>
-        </is>
-      </c>
-      <c r="E32" s="47">
-        <f>'L. VENTAS'!P19</f>
+          <t>Factura de venta N°104 a Comercial Maule SpA</t>
+        </is>
+      </c>
+      <c r="F32" s="47">
+        <f>'L. VENTAS'!H9</f>
         <v/>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>11</v>
-      </c>
-      <c r="B33" s="421" t="n">
-        <v>46326</v>
+        <v>9</v>
+      </c>
+      <c r="B33" s="420" t="n">
+        <v>46316</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>1.1.13 Inventario mercaderías</t>
+          <t>2.1.02 IVA débito fiscal</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Costo de las ventas del mes</t>
+          <t>Factura de venta N°104 a Comercial Maule SpA</t>
         </is>
       </c>
       <c r="F33" s="47">
-        <f>'L. VENTAS'!P19</f>
+        <f>'L. VENTAS'!I9</f>
         <v/>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>12</v>
-      </c>
-      <c r="B34" s="421" t="n">
-        <v>46326</v>
+        <v>10</v>
+      </c>
+      <c r="B34" s="420" t="n">
+        <v>46323</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>2.1.01 Proveedores</t>
+          <t>1.1.03 Clientes</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Pago a los proveedores</t>
+          <t>Factura de venta N°105 a Distribuidora Bío Bío Ltda.</t>
         </is>
       </c>
       <c r="E34" s="47">
-        <f>'L. COMPRAS'!O16</f>
+        <f>'L. VENTAS'!J10</f>
         <v/>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>12</v>
-      </c>
-      <c r="B35" s="421" t="n">
-        <v>46326</v>
+        <v>10</v>
+      </c>
+      <c r="B35" s="420" t="n">
+        <v>46323</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>1.1.02 Banco</t>
+          <t>4.1.01 Ventas</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Pago a los proveedores</t>
+          <t>Factura de venta N°105 a Distribuidora Bío Bío Ltda.</t>
         </is>
       </c>
       <c r="F35" s="47">
-        <f>'L. COMPRAS'!O16</f>
+        <f>'L. VENTAS'!H10</f>
         <v/>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>13</v>
-      </c>
-      <c r="B36" s="421" t="n">
-        <v>46338</v>
+        <v>10</v>
+      </c>
+      <c r="B36" s="420" t="n">
+        <v>46323</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -12906,96 +12905,228 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>F29: débito, IVA retenido y PPM</t>
-        </is>
-      </c>
-      <c r="E36" s="47">
-        <f>'FORMULARIO 29'!AP16</f>
+          <t>Factura de venta N°105 a Distribuidora Bío Bío Ltda.</t>
+        </is>
+      </c>
+      <c r="F36" s="47">
+        <f>'L. VENTAS'!I10</f>
         <v/>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>13</v>
-      </c>
-      <c r="B37" s="421" t="n">
-        <v>46338</v>
+        <v>11</v>
+      </c>
+      <c r="B37" s="420" t="n">
+        <v>46326</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>2.1.09 IVA retenido por pagar</t>
+          <t>5.1.01 Costo de ventas</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>F29: débito, IVA retenido y PPM</t>
+          <t>Costo de las ventas del mes</t>
         </is>
       </c>
       <c r="E37" s="47">
-        <f>'FORMULARIO 29'!AP97</f>
+        <f>'L. VENTAS'!P19</f>
         <v/>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>13</v>
-      </c>
-      <c r="B38" s="421" t="n">
-        <v>46338</v>
+        <v>11</v>
+      </c>
+      <c r="B38" s="420" t="n">
+        <v>46326</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>1.1.05 PPM por recuperar</t>
+          <t>1.1.13 Inventario mercaderías</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>F29: débito, IVA retenido y PPM</t>
-        </is>
-      </c>
-      <c r="E38" s="47">
-        <f>'FORMULARIO 29'!AP74</f>
+          <t>Costo de las ventas del mes</t>
+        </is>
+      </c>
+      <c r="F38" s="47">
+        <f>'L. VENTAS'!P19</f>
         <v/>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
+        <v>12</v>
+      </c>
+      <c r="B39" s="420" t="n">
+        <v>46326</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>2.1.01 Proveedores</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Pago a los proveedores</t>
+        </is>
+      </c>
+      <c r="E39" s="47">
+        <f>'L. COMPRAS'!O16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>12</v>
+      </c>
+      <c r="B40" s="420" t="n">
+        <v>46326</v>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>1.1.02 Banco</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Pago a los proveedores</t>
+        </is>
+      </c>
+      <c r="F40" s="47">
+        <f>'L. COMPRAS'!O16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
         <v>13</v>
       </c>
-      <c r="B39" s="421" t="n">
+      <c r="B41" s="420" t="n">
         <v>46338</v>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>2.1.02 IVA débito fiscal</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>F29: débito menos crédito, IVA retenido y PPM</t>
+        </is>
+      </c>
+      <c r="E41" s="47">
+        <f>'FORMULARIO 29'!AP16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>13</v>
+      </c>
+      <c r="B42" s="420" t="n">
+        <v>46338</v>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>2.1.09 IVA retenido por pagar</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>F29: débito menos crédito, IVA retenido y PPM</t>
+        </is>
+      </c>
+      <c r="E42" s="47">
+        <f>'FORMULARIO 29'!AP97</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>13</v>
+      </c>
+      <c r="B43" s="420" t="n">
+        <v>46338</v>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>1.1.05 PPM por recuperar</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>F29: débito menos crédito, IVA retenido y PPM</t>
+        </is>
+      </c>
+      <c r="E43" s="47">
+        <f>'FORMULARIO 29'!AP74</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>13</v>
+      </c>
+      <c r="B44" s="420" t="n">
+        <v>46338</v>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>1.1.04 IVA crédito fiscal</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>F29: débito menos crédito, IVA retenido y PPM</t>
+        </is>
+      </c>
+      <c r="F44" s="47">
+        <f>'FORMULARIO 29'!AP58</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>13</v>
+      </c>
+      <c r="B45" s="420" t="n">
+        <v>46338</v>
+      </c>
+      <c r="C45" t="inlineStr">
         <is>
           <t>1.1.02 Banco</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>F29: débito, IVA retenido y PPM</t>
-        </is>
-      </c>
-      <c r="F39" s="47">
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>F29: débito menos crédito, IVA retenido y PPM</t>
+        </is>
+      </c>
+      <c r="F45" s="47">
         <f>'FORMULARIO 29'!AP92</f>
         <v/>
       </c>
     </row>
-    <row r="40">
-      <c r="D40" s="336" t="inlineStr">
+    <row r="46">
+      <c r="D46" s="336" t="inlineStr">
         <is>
           <t>SUMAS IGUALES</t>
         </is>
       </c>
-      <c r="E40" s="47">
-        <f>SUM(E2:E39)</f>
-        <v/>
-      </c>
-      <c r="F40" s="47">
-        <f>SUM(F2:F39)</f>
-        <v/>
-      </c>
-      <c r="G40">
-        <f>IF(E40=F40,"Cuadra","NO CUADRA")</f>
+      <c r="E46" s="47">
+        <f>SUM(E2:E45)</f>
+        <v/>
+      </c>
+      <c r="F46" s="47">
+        <f>SUM(F2:F45)</f>
+        <v/>
+      </c>
+      <c r="G46">
+        <f>IF(E46=F46,"Cuadra","NO CUADRA")</f>
         <v/>
       </c>
     </row>
@@ -13039,47 +13170,47 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="417" t="inlineStr">
+      <c r="A4" s="416" t="inlineStr">
         <is>
           <t>RUT del vendedor (retenido)</t>
         </is>
       </c>
-      <c r="B4" s="417" t="inlineStr">
+      <c r="B4" s="416" t="inlineStr">
         <is>
           <t>Código de producto (F3500)</t>
         </is>
       </c>
-      <c r="C4" s="417" t="inlineStr">
+      <c r="C4" s="416" t="inlineStr">
         <is>
           <t>Producto</t>
         </is>
       </c>
-      <c r="D4" s="417" t="inlineStr">
+      <c r="D4" s="416" t="inlineStr">
         <is>
           <t>Tipo de documento</t>
         </is>
       </c>
-      <c r="E4" s="417" t="inlineStr">
+      <c r="E4" s="416" t="inlineStr">
         <is>
           <t>N° documento</t>
         </is>
       </c>
-      <c r="F4" s="417" t="inlineStr">
+      <c r="F4" s="416" t="inlineStr">
         <is>
           <t>Fecha</t>
         </is>
       </c>
-      <c r="G4" s="417" t="inlineStr">
+      <c r="G4" s="416" t="inlineStr">
         <is>
           <t>Cantidad</t>
         </is>
       </c>
-      <c r="H4" s="417" t="inlineStr">
+      <c r="H4" s="416" t="inlineStr">
         <is>
           <t>Unidad de medida (cód. 1)</t>
         </is>
       </c>
-      <c r="I4" s="417" t="inlineStr">
+      <c r="I4" s="416" t="inlineStr">
         <is>
           <t>IVA retenido total</t>
         </is>
@@ -13107,7 +13238,7 @@
         <f>'L. COMPRAS'!B7</f>
         <v/>
       </c>
-      <c r="F5" s="421">
+      <c r="F5" s="420">
         <f>'L. COMPRAS'!A7</f>
         <v/>
       </c>
@@ -13145,7 +13276,7 @@
         <f>'L. COMPRAS'!B8</f>
         <v/>
       </c>
-      <c r="F6" s="421">
+      <c r="F6" s="420">
         <f>'L. COMPRAS'!A8</f>
         <v/>
       </c>
@@ -13183,7 +13314,7 @@
         <f>'L. COMPRAS'!B9</f>
         <v/>
       </c>
-      <c r="F7" s="421">
+      <c r="F7" s="420">
         <f>'L. COMPRAS'!A9</f>
         <v/>
       </c>
@@ -13221,7 +13352,7 @@
         <f>'L. COMPRAS'!B10</f>
         <v/>
       </c>
-      <c r="F8" s="421">
+      <c r="F8" s="420">
         <f>'L. COMPRAS'!A10</f>
         <v/>
       </c>
@@ -13259,7 +13390,7 @@
         <f>'L. COMPRAS'!B11</f>
         <v/>
       </c>
-      <c r="F9" s="421">
+      <c r="F9" s="420">
         <f>'L. COMPRAS'!A11</f>
         <v/>
       </c>

</xml_diff>